<commit_message>
feat: Update FastAPI backend to use port 8001 and adjust Nginx configuration
- Changed FastAPI backend to run on port 8001 instead of 8000.
- Updated Nginx configuration to proxy API requests to the new backend port.
- Modified run.bat script to reflect the new backend port.
- Enhanced data model to specify custom_config as a list of dictionaries.
- Updated workload configuration to reflect new asset definitions and unit costs.
- Implemented caching for data loading functions to improve performance.
- Added a new script to insert a 'bridge_m' column into the Excel data file.
</commit_message>
<xml_diff>
--- a/data/group_data_final.xlsx
+++ b/data/group_data_final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://infracorpth-my.sharepoint.com/personal/inthat_l_infra-corp_co/Documents/rmms/WL/webapp/workload_webapp/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{3FAAEDA8-C7EE-439B-AB68-C2F6B5CF4980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{668E017B-77B0-4B20-BDFF-A163B7AD1839}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{21ACC0D1-E520-4769-8E42-7F4F5CC34E5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{06DD2867-C549-4802-9494-1CB8AE5F8E10}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{06DD2867-C549-4802-9494-1CB8AE5F8E10}"/>
   </bookViews>
   <sheets>
     <sheet name="group_data_final" sheetId="2" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1656" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1657" uniqueCount="531">
   <si>
     <t>division_name</t>
   </si>
@@ -1668,6 +1668,9 @@
   <si>
     <t>veh_truck</t>
   </si>
+  <si>
+    <t>bridge_m</t>
+  </si>
 </sst>
 </file>
 
@@ -2515,7 +2518,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="35" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2710,12 +2713,6 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="33" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2728,7 +2725,12 @@
     <xf numFmtId="0" fontId="22" fillId="33" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -3330,7 +3332,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E98ED939-3D95-436D-AB62-CAD7A9B06D1A}">
-  <dimension ref="A1:AM105"/>
+  <dimension ref="A1:AN105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="37.140625" bestFit="1" customWidth="1"/>
@@ -3371,7 +3373,7 @@
     <col min="39" max="39" width="29.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39">
+    <row r="1" spans="1:40">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3489,8 +3491,11 @@
       <c r="AM1" t="s">
         <v>521</v>
       </c>
-    </row>
-    <row r="2" spans="1:39">
+      <c r="AN1" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="2" spans="1:40">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -3613,7 +3618,7 @@
         <v>0</v>
       </c>
       <c r="AL2">
-        <f>IF(OR(COUNTIF(B2,"*กระบี่*"),COUNTIF(B2,"*จันทบุรี*"),COUNTIF(B2,"*ชุมพร*"),COUNTIF(B2,"*เชียงราย*"),COUNTIF(B2,"*ตรัง*"),COUNTIF(B2,"*นครนายก*"),COUNTIF(B2,"*ปราจีนบุรี*"),COUNTIF(B2,"*พัทลุง*"),COUNTIF(B2,"*ภูเก็ต*"),COUNTIF(B2,"*ยะลา*"),COUNTIF(B2,"*สกลนคร*"),COUNTIF(B2,"*สตูล*"),COUNTIF(B2,"*หนองคาย*"),COUNTIF(B2,"*สุราษฎร์ธานี*"),COUNTIF(B2,"*ปัตตานี*")),2,
+        <f t="shared" ref="AL2:AL33" si="0">IF(OR(COUNTIF(B2,"*กระบี่*"),COUNTIF(B2,"*จันทบุรี*"),COUNTIF(B2,"*ชุมพร*"),COUNTIF(B2,"*เชียงราย*"),COUNTIF(B2,"*ตรัง*"),COUNTIF(B2,"*นครนายก*"),COUNTIF(B2,"*ปราจีนบุรี*"),COUNTIF(B2,"*พัทลุง*"),COUNTIF(B2,"*ภูเก็ต*"),COUNTIF(B2,"*ยะลา*"),COUNTIF(B2,"*สกลนคร*"),COUNTIF(B2,"*สตูล*"),COUNTIF(B2,"*หนองคาย*"),COUNTIF(B2,"*สุราษฎร์ธานี*"),COUNTIF(B2,"*ปัตตานี*")),2,
 IF(OR(COUNTIF(B2,"*ตราด*"),COUNTIF(B2,"*นครพนม*"),COUNTIF(B2,"*นครศรีธรรมราช*"),COUNTIF(B2,"*นราธิวาส*"),COUNTIF(B2,"*บึงกาฬ*"),COUNTIF(B2,"*พังงา*"),COUNTIF(B2,"*ระนอง*"),COUNTIF(B2,"*สงขลา*")),4,0))</f>
         <v>4</v>
       </c>
@@ -3621,8 +3626,11 @@
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>20573476</v>
       </c>
-    </row>
-    <row r="3" spans="1:39" s="32" customFormat="1" ht="24">
+      <c r="AN2">
+        <v>17246.601999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:40" s="32" customFormat="1" ht="24">
       <c r="A3" s="32" t="s">
         <v>37</v>
       </c>
@@ -3745,16 +3753,18 @@
         <v>900000</v>
       </c>
       <c r="AL3" s="32">
-        <f>IF(OR(COUNTIF(B3,"*กระบี่*"),COUNTIF(B3,"*จันทบุรี*"),COUNTIF(B3,"*ชุมพร*"),COUNTIF(B3,"*เชียงราย*"),COUNTIF(B3,"*ตรัง*"),COUNTIF(B3,"*นครนายก*"),COUNTIF(B3,"*ปราจีนบุรี*"),COUNTIF(B3,"*พัทลุง*"),COUNTIF(B3,"*ภูเก็ต*"),COUNTIF(B3,"*ยะลา*"),COUNTIF(B3,"*สกลนคร*"),COUNTIF(B3,"*สตูล*"),COUNTIF(B3,"*หนองคาย*"),COUNTIF(B3,"*สุราษฎร์ธานี*"),COUNTIF(B3,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B3,"*ตราด*"),COUNTIF(B3,"*นครพนม*"),COUNTIF(B3,"*นครศรีธรรมราช*"),COUNTIF(B3,"*นราธิวาส*"),COUNTIF(B3,"*บึงกาฬ*"),COUNTIF(B3,"*พังงา*"),COUNTIF(B3,"*ระนอง*"),COUNTIF(B3,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM3">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>24198050.16</v>
       </c>
-    </row>
-    <row r="4" spans="1:39" s="32" customFormat="1" ht="24">
+      <c r="AN3">
+        <v>7504</v>
+      </c>
+    </row>
+    <row r="4" spans="1:40" s="32" customFormat="1" ht="24">
       <c r="A4" s="32" t="s">
         <v>37</v>
       </c>
@@ -3877,16 +3887,18 @@
         <v>0</v>
       </c>
       <c r="AL4" s="32">
-        <f>IF(OR(COUNTIF(B4,"*กระบี่*"),COUNTIF(B4,"*จันทบุรี*"),COUNTIF(B4,"*ชุมพร*"),COUNTIF(B4,"*เชียงราย*"),COUNTIF(B4,"*ตรัง*"),COUNTIF(B4,"*นครนายก*"),COUNTIF(B4,"*ปราจีนบุรี*"),COUNTIF(B4,"*พัทลุง*"),COUNTIF(B4,"*ภูเก็ต*"),COUNTIF(B4,"*ยะลา*"),COUNTIF(B4,"*สกลนคร*"),COUNTIF(B4,"*สตูล*"),COUNTIF(B4,"*หนองคาย*"),COUNTIF(B4,"*สุราษฎร์ธานี*"),COUNTIF(B4,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B4,"*ตราด*"),COUNTIF(B4,"*นครพนม*"),COUNTIF(B4,"*นครศรีธรรมราช*"),COUNTIF(B4,"*นราธิวาส*"),COUNTIF(B4,"*บึงกาฬ*"),COUNTIF(B4,"*พังงา*"),COUNTIF(B4,"*ระนอง*"),COUNTIF(B4,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM4">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>56319717.350000001</v>
       </c>
-    </row>
-    <row r="5" spans="1:39">
+      <c r="AN4">
+        <v>13095.525</v>
+      </c>
+    </row>
+    <row r="5" spans="1:40">
       <c r="A5" t="s">
         <v>41</v>
       </c>
@@ -4009,16 +4021,18 @@
         <v>0</v>
       </c>
       <c r="AL5">
-        <f>IF(OR(COUNTIF(B5,"*กระบี่*"),COUNTIF(B5,"*จันทบุรี*"),COUNTIF(B5,"*ชุมพร*"),COUNTIF(B5,"*เชียงราย*"),COUNTIF(B5,"*ตรัง*"),COUNTIF(B5,"*นครนายก*"),COUNTIF(B5,"*ปราจีนบุรี*"),COUNTIF(B5,"*พัทลุง*"),COUNTIF(B5,"*ภูเก็ต*"),COUNTIF(B5,"*ยะลา*"),COUNTIF(B5,"*สกลนคร*"),COUNTIF(B5,"*สตูล*"),COUNTIF(B5,"*หนองคาย*"),COUNTIF(B5,"*สุราษฎร์ธานี*"),COUNTIF(B5,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B5,"*ตราด*"),COUNTIF(B5,"*นครพนม*"),COUNTIF(B5,"*นครศรีธรรมราช*"),COUNTIF(B5,"*นราธิวาส*"),COUNTIF(B5,"*บึงกาฬ*"),COUNTIF(B5,"*พังงา*"),COUNTIF(B5,"*ระนอง*"),COUNTIF(B5,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM5">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>16076823.02</v>
       </c>
-    </row>
-    <row r="6" spans="1:39" s="32" customFormat="1" ht="24">
+      <c r="AN5">
+        <v>7998.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:40" s="32" customFormat="1" ht="24">
       <c r="A6" s="32" t="s">
         <v>37</v>
       </c>
@@ -4141,16 +4155,18 @@
         <v>0</v>
       </c>
       <c r="AL6" s="32">
-        <f>IF(OR(COUNTIF(B6,"*กระบี่*"),COUNTIF(B6,"*จันทบุรี*"),COUNTIF(B6,"*ชุมพร*"),COUNTIF(B6,"*เชียงราย*"),COUNTIF(B6,"*ตรัง*"),COUNTIF(B6,"*นครนายก*"),COUNTIF(B6,"*ปราจีนบุรี*"),COUNTIF(B6,"*พัทลุง*"),COUNTIF(B6,"*ภูเก็ต*"),COUNTIF(B6,"*ยะลา*"),COUNTIF(B6,"*สกลนคร*"),COUNTIF(B6,"*สตูล*"),COUNTIF(B6,"*หนองคาย*"),COUNTIF(B6,"*สุราษฎร์ธานี*"),COUNTIF(B6,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B6,"*ตราด*"),COUNTIF(B6,"*นครพนม*"),COUNTIF(B6,"*นครศรีธรรมราช*"),COUNTIF(B6,"*นราธิวาส*"),COUNTIF(B6,"*บึงกาฬ*"),COUNTIF(B6,"*พังงา*"),COUNTIF(B6,"*ระนอง*"),COUNTIF(B6,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="AM6">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>38452908.219999999</v>
       </c>
-    </row>
-    <row r="7" spans="1:39">
+      <c r="AN6">
+        <v>14423.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:40">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -4273,16 +4289,18 @@
         <v>0</v>
       </c>
       <c r="AL7">
-        <f>IF(OR(COUNTIF(B7,"*กระบี่*"),COUNTIF(B7,"*จันทบุรี*"),COUNTIF(B7,"*ชุมพร*"),COUNTIF(B7,"*เชียงราย*"),COUNTIF(B7,"*ตรัง*"),COUNTIF(B7,"*นครนายก*"),COUNTIF(B7,"*ปราจีนบุรี*"),COUNTIF(B7,"*พัทลุง*"),COUNTIF(B7,"*ภูเก็ต*"),COUNTIF(B7,"*ยะลา*"),COUNTIF(B7,"*สกลนคร*"),COUNTIF(B7,"*สตูล*"),COUNTIF(B7,"*หนองคาย*"),COUNTIF(B7,"*สุราษฎร์ธานี*"),COUNTIF(B7,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B7,"*ตราด*"),COUNTIF(B7,"*นครพนม*"),COUNTIF(B7,"*นครศรีธรรมราช*"),COUNTIF(B7,"*นราธิวาส*"),COUNTIF(B7,"*บึงกาฬ*"),COUNTIF(B7,"*พังงา*"),COUNTIF(B7,"*ระนอง*"),COUNTIF(B7,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM7">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>35219242</v>
       </c>
-    </row>
-    <row r="8" spans="1:39" s="32" customFormat="1" ht="24">
+      <c r="AN7">
+        <v>2927</v>
+      </c>
+    </row>
+    <row r="8" spans="1:40" s="32" customFormat="1" ht="24">
       <c r="A8" s="32" t="s">
         <v>37</v>
       </c>
@@ -4405,16 +4423,18 @@
         <v>0</v>
       </c>
       <c r="AL8" s="32">
-        <f>IF(OR(COUNTIF(B8,"*กระบี่*"),COUNTIF(B8,"*จันทบุรี*"),COUNTIF(B8,"*ชุมพร*"),COUNTIF(B8,"*เชียงราย*"),COUNTIF(B8,"*ตรัง*"),COUNTIF(B8,"*นครนายก*"),COUNTIF(B8,"*ปราจีนบุรี*"),COUNTIF(B8,"*พัทลุง*"),COUNTIF(B8,"*ภูเก็ต*"),COUNTIF(B8,"*ยะลา*"),COUNTIF(B8,"*สกลนคร*"),COUNTIF(B8,"*สตูล*"),COUNTIF(B8,"*หนองคาย*"),COUNTIF(B8,"*สุราษฎร์ธานี*"),COUNTIF(B8,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B8,"*ตราด*"),COUNTIF(B8,"*นครพนม*"),COUNTIF(B8,"*นครศรีธรรมราช*"),COUNTIF(B8,"*นราธิวาส*"),COUNTIF(B8,"*บึงกาฬ*"),COUNTIF(B8,"*พังงา*"),COUNTIF(B8,"*ระนอง*"),COUNTIF(B8,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="AM8">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>15992685.75</v>
       </c>
-    </row>
-    <row r="9" spans="1:39">
+      <c r="AN8">
+        <v>5798.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:40">
       <c r="A9" t="s">
         <v>41</v>
       </c>
@@ -4537,16 +4557,18 @@
         <v>0</v>
       </c>
       <c r="AL9">
-        <f>IF(OR(COUNTIF(B9,"*กระบี่*"),COUNTIF(B9,"*จันทบุรี*"),COUNTIF(B9,"*ชุมพร*"),COUNTIF(B9,"*เชียงราย*"),COUNTIF(B9,"*ตรัง*"),COUNTIF(B9,"*นครนายก*"),COUNTIF(B9,"*ปราจีนบุรี*"),COUNTIF(B9,"*พัทลุง*"),COUNTIF(B9,"*ภูเก็ต*"),COUNTIF(B9,"*ยะลา*"),COUNTIF(B9,"*สกลนคร*"),COUNTIF(B9,"*สตูล*"),COUNTIF(B9,"*หนองคาย*"),COUNTIF(B9,"*สุราษฎร์ธานี*"),COUNTIF(B9,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B9,"*ตราด*"),COUNTIF(B9,"*นครพนม*"),COUNTIF(B9,"*นครศรีธรรมราช*"),COUNTIF(B9,"*นราธิวาส*"),COUNTIF(B9,"*บึงกาฬ*"),COUNTIF(B9,"*พังงา*"),COUNTIF(B9,"*ระนอง*"),COUNTIF(B9,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="AM9">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>20146537</v>
       </c>
-    </row>
-    <row r="10" spans="1:39">
+      <c r="AN9">
+        <v>16169.3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:40">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -4669,16 +4691,18 @@
         <v>0</v>
       </c>
       <c r="AL10">
-        <f>IF(OR(COUNTIF(B10,"*กระบี่*"),COUNTIF(B10,"*จันทบุรี*"),COUNTIF(B10,"*ชุมพร*"),COUNTIF(B10,"*เชียงราย*"),COUNTIF(B10,"*ตรัง*"),COUNTIF(B10,"*นครนายก*"),COUNTIF(B10,"*ปราจีนบุรี*"),COUNTIF(B10,"*พัทลุง*"),COUNTIF(B10,"*ภูเก็ต*"),COUNTIF(B10,"*ยะลา*"),COUNTIF(B10,"*สกลนคร*"),COUNTIF(B10,"*สตูล*"),COUNTIF(B10,"*หนองคาย*"),COUNTIF(B10,"*สุราษฎร์ธานี*"),COUNTIF(B10,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B10,"*ตราด*"),COUNTIF(B10,"*นครพนม*"),COUNTIF(B10,"*นครศรีธรรมราช*"),COUNTIF(B10,"*นราธิวาส*"),COUNTIF(B10,"*บึงกาฬ*"),COUNTIF(B10,"*พังงา*"),COUNTIF(B10,"*ระนอง*"),COUNTIF(B10,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM10">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>13871166.91</v>
       </c>
-    </row>
-    <row r="11" spans="1:39">
+      <c r="AN10">
+        <v>7842.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:40">
       <c r="A11" t="s">
         <v>47</v>
       </c>
@@ -4795,16 +4819,18 @@
         <v>1500000</v>
       </c>
       <c r="AL11">
-        <f>IF(OR(COUNTIF(B11,"*กระบี่*"),COUNTIF(B11,"*จันทบุรี*"),COUNTIF(B11,"*ชุมพร*"),COUNTIF(B11,"*เชียงราย*"),COUNTIF(B11,"*ตรัง*"),COUNTIF(B11,"*นครนายก*"),COUNTIF(B11,"*ปราจีนบุรี*"),COUNTIF(B11,"*พัทลุง*"),COUNTIF(B11,"*ภูเก็ต*"),COUNTIF(B11,"*ยะลา*"),COUNTIF(B11,"*สกลนคร*"),COUNTIF(B11,"*สตูล*"),COUNTIF(B11,"*หนองคาย*"),COUNTIF(B11,"*สุราษฎร์ธานี*"),COUNTIF(B11,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B11,"*ตราด*"),COUNTIF(B11,"*นครพนม*"),COUNTIF(B11,"*นครศรีธรรมราช*"),COUNTIF(B11,"*นราธิวาส*"),COUNTIF(B11,"*บึงกาฬ*"),COUNTIF(B11,"*พังงา*"),COUNTIF(B11,"*ระนอง*"),COUNTIF(B11,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM11">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>9306767.8200000003</v>
       </c>
-    </row>
-    <row r="12" spans="1:39">
+      <c r="AN11">
+        <v>4899.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:40">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -4927,16 +4953,18 @@
         <v>600000</v>
       </c>
       <c r="AL12">
-        <f>IF(OR(COUNTIF(B12,"*กระบี่*"),COUNTIF(B12,"*จันทบุรี*"),COUNTIF(B12,"*ชุมพร*"),COUNTIF(B12,"*เชียงราย*"),COUNTIF(B12,"*ตรัง*"),COUNTIF(B12,"*นครนายก*"),COUNTIF(B12,"*ปราจีนบุรี*"),COUNTIF(B12,"*พัทลุง*"),COUNTIF(B12,"*ภูเก็ต*"),COUNTIF(B12,"*ยะลา*"),COUNTIF(B12,"*สกลนคร*"),COUNTIF(B12,"*สตูล*"),COUNTIF(B12,"*หนองคาย*"),COUNTIF(B12,"*สุราษฎร์ธานี*"),COUNTIF(B12,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B12,"*ตราด*"),COUNTIF(B12,"*นครพนม*"),COUNTIF(B12,"*นครศรีธรรมราช*"),COUNTIF(B12,"*นราธิวาส*"),COUNTIF(B12,"*บึงกาฬ*"),COUNTIF(B12,"*พังงา*"),COUNTIF(B12,"*ระนอง*"),COUNTIF(B12,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM12">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>17236877.359999999</v>
       </c>
-    </row>
-    <row r="13" spans="1:39">
+      <c r="AN12">
+        <v>3881.05</v>
+      </c>
+    </row>
+    <row r="13" spans="1:40">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -5059,16 +5087,18 @@
         <v>0</v>
       </c>
       <c r="AL13">
-        <f>IF(OR(COUNTIF(B13,"*กระบี่*"),COUNTIF(B13,"*จันทบุรี*"),COUNTIF(B13,"*ชุมพร*"),COUNTIF(B13,"*เชียงราย*"),COUNTIF(B13,"*ตรัง*"),COUNTIF(B13,"*นครนายก*"),COUNTIF(B13,"*ปราจีนบุรี*"),COUNTIF(B13,"*พัทลุง*"),COUNTIF(B13,"*ภูเก็ต*"),COUNTIF(B13,"*ยะลา*"),COUNTIF(B13,"*สกลนคร*"),COUNTIF(B13,"*สตูล*"),COUNTIF(B13,"*หนองคาย*"),COUNTIF(B13,"*สุราษฎร์ธานี*"),COUNTIF(B13,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B13,"*ตราด*"),COUNTIF(B13,"*นครพนม*"),COUNTIF(B13,"*นครศรีธรรมราช*"),COUNTIF(B13,"*นราธิวาส*"),COUNTIF(B13,"*บึงกาฬ*"),COUNTIF(B13,"*พังงา*"),COUNTIF(B13,"*ระนอง*"),COUNTIF(B13,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM13">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>47805316</v>
       </c>
-    </row>
-    <row r="14" spans="1:39">
+      <c r="AN13">
+        <v>19521.95</v>
+      </c>
+    </row>
+    <row r="14" spans="1:40">
       <c r="A14" t="s">
         <v>41</v>
       </c>
@@ -5188,16 +5218,18 @@
         <v>600000</v>
       </c>
       <c r="AL14">
-        <f>IF(OR(COUNTIF(B14,"*กระบี่*"),COUNTIF(B14,"*จันทบุรี*"),COUNTIF(B14,"*ชุมพร*"),COUNTIF(B14,"*เชียงราย*"),COUNTIF(B14,"*ตรัง*"),COUNTIF(B14,"*นครนายก*"),COUNTIF(B14,"*ปราจีนบุรี*"),COUNTIF(B14,"*พัทลุง*"),COUNTIF(B14,"*ภูเก็ต*"),COUNTIF(B14,"*ยะลา*"),COUNTIF(B14,"*สกลนคร*"),COUNTIF(B14,"*สตูล*"),COUNTIF(B14,"*หนองคาย*"),COUNTIF(B14,"*สุราษฎร์ธานี*"),COUNTIF(B14,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B14,"*ตราด*"),COUNTIF(B14,"*นครพนม*"),COUNTIF(B14,"*นครศรีธรรมราช*"),COUNTIF(B14,"*นราธิวาส*"),COUNTIF(B14,"*บึงกาฬ*"),COUNTIF(B14,"*พังงา*"),COUNTIF(B14,"*ระนอง*"),COUNTIF(B14,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="AM14">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>46419930</v>
       </c>
-    </row>
-    <row r="15" spans="1:39">
+      <c r="AN14">
+        <v>10490.415000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:40">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -5320,16 +5352,18 @@
         <v>0</v>
       </c>
       <c r="AL15">
-        <f>IF(OR(COUNTIF(B15,"*กระบี่*"),COUNTIF(B15,"*จันทบุรี*"),COUNTIF(B15,"*ชุมพร*"),COUNTIF(B15,"*เชียงราย*"),COUNTIF(B15,"*ตรัง*"),COUNTIF(B15,"*นครนายก*"),COUNTIF(B15,"*ปราจีนบุรี*"),COUNTIF(B15,"*พัทลุง*"),COUNTIF(B15,"*ภูเก็ต*"),COUNTIF(B15,"*ยะลา*"),COUNTIF(B15,"*สกลนคร*"),COUNTIF(B15,"*สตูล*"),COUNTIF(B15,"*หนองคาย*"),COUNTIF(B15,"*สุราษฎร์ธานี*"),COUNTIF(B15,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B15,"*ตราด*"),COUNTIF(B15,"*นครพนม*"),COUNTIF(B15,"*นครศรีธรรมราช*"),COUNTIF(B15,"*นราธิวาส*"),COUNTIF(B15,"*บึงกาฬ*"),COUNTIF(B15,"*พังงา*"),COUNTIF(B15,"*ระนอง*"),COUNTIF(B15,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="AM15">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>22852169.210000001</v>
       </c>
-    </row>
-    <row r="16" spans="1:39">
+      <c r="AN15">
+        <v>9585.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:40">
       <c r="A16" t="s">
         <v>41</v>
       </c>
@@ -5437,16 +5471,18 @@
         <v>300000</v>
       </c>
       <c r="AL16">
-        <f>IF(OR(COUNTIF(B16,"*กระบี่*"),COUNTIF(B16,"*จันทบุรี*"),COUNTIF(B16,"*ชุมพร*"),COUNTIF(B16,"*เชียงราย*"),COUNTIF(B16,"*ตรัง*"),COUNTIF(B16,"*นครนายก*"),COUNTIF(B16,"*ปราจีนบุรี*"),COUNTIF(B16,"*พัทลุง*"),COUNTIF(B16,"*ภูเก็ต*"),COUNTIF(B16,"*ยะลา*"),COUNTIF(B16,"*สกลนคร*"),COUNTIF(B16,"*สตูล*"),COUNTIF(B16,"*หนองคาย*"),COUNTIF(B16,"*สุราษฎร์ธานี*"),COUNTIF(B16,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B16,"*ตราด*"),COUNTIF(B16,"*นครพนม*"),COUNTIF(B16,"*นครศรีธรรมราช*"),COUNTIF(B16,"*นราธิวาส*"),COUNTIF(B16,"*บึงกาฬ*"),COUNTIF(B16,"*พังงา*"),COUNTIF(B16,"*ระนอง*"),COUNTIF(B16,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM16">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>26661755.600000001</v>
       </c>
-    </row>
-    <row r="17" spans="1:39">
+      <c r="AN16">
+        <v>8649</v>
+      </c>
+    </row>
+    <row r="17" spans="1:40">
       <c r="A17" t="s">
         <v>41</v>
       </c>
@@ -5563,16 +5599,18 @@
         <v>0</v>
       </c>
       <c r="AL17">
-        <f>IF(OR(COUNTIF(B17,"*กระบี่*"),COUNTIF(B17,"*จันทบุรี*"),COUNTIF(B17,"*ชุมพร*"),COUNTIF(B17,"*เชียงราย*"),COUNTIF(B17,"*ตรัง*"),COUNTIF(B17,"*นครนายก*"),COUNTIF(B17,"*ปราจีนบุรี*"),COUNTIF(B17,"*พัทลุง*"),COUNTIF(B17,"*ภูเก็ต*"),COUNTIF(B17,"*ยะลา*"),COUNTIF(B17,"*สกลนคร*"),COUNTIF(B17,"*สตูล*"),COUNTIF(B17,"*หนองคาย*"),COUNTIF(B17,"*สุราษฎร์ธานี*"),COUNTIF(B17,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B17,"*ตราด*"),COUNTIF(B17,"*นครพนม*"),COUNTIF(B17,"*นครศรีธรรมราช*"),COUNTIF(B17,"*นราธิวาส*"),COUNTIF(B17,"*บึงกาฬ*"),COUNTIF(B17,"*พังงา*"),COUNTIF(B17,"*ระนอง*"),COUNTIF(B17,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM17">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>49094616.020000003</v>
       </c>
-    </row>
-    <row r="18" spans="1:39">
+      <c r="AN17">
+        <v>7855</v>
+      </c>
+    </row>
+    <row r="18" spans="1:40">
       <c r="A18" t="s">
         <v>47</v>
       </c>
@@ -5689,16 +5727,18 @@
         <v>0</v>
       </c>
       <c r="AL18">
-        <f>IF(OR(COUNTIF(B18,"*กระบี่*"),COUNTIF(B18,"*จันทบุรี*"),COUNTIF(B18,"*ชุมพร*"),COUNTIF(B18,"*เชียงราย*"),COUNTIF(B18,"*ตรัง*"),COUNTIF(B18,"*นครนายก*"),COUNTIF(B18,"*ปราจีนบุรี*"),COUNTIF(B18,"*พัทลุง*"),COUNTIF(B18,"*ภูเก็ต*"),COUNTIF(B18,"*ยะลา*"),COUNTIF(B18,"*สกลนคร*"),COUNTIF(B18,"*สตูล*"),COUNTIF(B18,"*หนองคาย*"),COUNTIF(B18,"*สุราษฎร์ธานี*"),COUNTIF(B18,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B18,"*ตราด*"),COUNTIF(B18,"*นครพนม*"),COUNTIF(B18,"*นครศรีธรรมราช*"),COUNTIF(B18,"*นราธิวาส*"),COUNTIF(B18,"*บึงกาฬ*"),COUNTIF(B18,"*พังงา*"),COUNTIF(B18,"*ระนอง*"),COUNTIF(B18,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="AM18">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>35764703</v>
       </c>
-    </row>
-    <row r="19" spans="1:39">
+      <c r="AN18">
+        <v>7390</v>
+      </c>
+    </row>
+    <row r="19" spans="1:40">
       <c r="A19" t="s">
         <v>57</v>
       </c>
@@ -5821,16 +5861,18 @@
         <v>0</v>
       </c>
       <c r="AL19">
-        <f>IF(OR(COUNTIF(B19,"*กระบี่*"),COUNTIF(B19,"*จันทบุรี*"),COUNTIF(B19,"*ชุมพร*"),COUNTIF(B19,"*เชียงราย*"),COUNTIF(B19,"*ตรัง*"),COUNTIF(B19,"*นครนายก*"),COUNTIF(B19,"*ปราจีนบุรี*"),COUNTIF(B19,"*พัทลุง*"),COUNTIF(B19,"*ภูเก็ต*"),COUNTIF(B19,"*ยะลา*"),COUNTIF(B19,"*สกลนคร*"),COUNTIF(B19,"*สตูล*"),COUNTIF(B19,"*หนองคาย*"),COUNTIF(B19,"*สุราษฎร์ธานี*"),COUNTIF(B19,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B19,"*ตราด*"),COUNTIF(B19,"*นครพนม*"),COUNTIF(B19,"*นครศรีธรรมราช*"),COUNTIF(B19,"*นราธิวาส*"),COUNTIF(B19,"*บึงกาฬ*"),COUNTIF(B19,"*พังงา*"),COUNTIF(B19,"*ระนอง*"),COUNTIF(B19,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM19">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>17220342</v>
       </c>
-    </row>
-    <row r="20" spans="1:39">
+      <c r="AN19">
+        <v>8576</v>
+      </c>
+    </row>
+    <row r="20" spans="1:40">
       <c r="A20" t="s">
         <v>57</v>
       </c>
@@ -5953,16 +5995,18 @@
         <v>0</v>
       </c>
       <c r="AL20">
-        <f>IF(OR(COUNTIF(B20,"*กระบี่*"),COUNTIF(B20,"*จันทบุรี*"),COUNTIF(B20,"*ชุมพร*"),COUNTIF(B20,"*เชียงราย*"),COUNTIF(B20,"*ตรัง*"),COUNTIF(B20,"*นครนายก*"),COUNTIF(B20,"*ปราจีนบุรี*"),COUNTIF(B20,"*พัทลุง*"),COUNTIF(B20,"*ภูเก็ต*"),COUNTIF(B20,"*ยะลา*"),COUNTIF(B20,"*สกลนคร*"),COUNTIF(B20,"*สตูล*"),COUNTIF(B20,"*หนองคาย*"),COUNTIF(B20,"*สุราษฎร์ธานี*"),COUNTIF(B20,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B20,"*ตราด*"),COUNTIF(B20,"*นครพนม*"),COUNTIF(B20,"*นครศรีธรรมราช*"),COUNTIF(B20,"*นราธิวาส*"),COUNTIF(B20,"*บึงกาฬ*"),COUNTIF(B20,"*พังงา*"),COUNTIF(B20,"*ระนอง*"),COUNTIF(B20,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM20">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>43935646.859999999</v>
       </c>
-    </row>
-    <row r="21" spans="1:39">
+      <c r="AN20">
+        <v>6936.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:40">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -6085,16 +6129,18 @@
         <v>300000</v>
       </c>
       <c r="AL21">
-        <f>IF(OR(COUNTIF(B21,"*กระบี่*"),COUNTIF(B21,"*จันทบุรี*"),COUNTIF(B21,"*ชุมพร*"),COUNTIF(B21,"*เชียงราย*"),COUNTIF(B21,"*ตรัง*"),COUNTIF(B21,"*นครนายก*"),COUNTIF(B21,"*ปราจีนบุรี*"),COUNTIF(B21,"*พัทลุง*"),COUNTIF(B21,"*ภูเก็ต*"),COUNTIF(B21,"*ยะลา*"),COUNTIF(B21,"*สกลนคร*"),COUNTIF(B21,"*สตูล*"),COUNTIF(B21,"*หนองคาย*"),COUNTIF(B21,"*สุราษฎร์ธานี*"),COUNTIF(B21,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B21,"*ตราด*"),COUNTIF(B21,"*นครพนม*"),COUNTIF(B21,"*นครศรีธรรมราช*"),COUNTIF(B21,"*นราธิวาส*"),COUNTIF(B21,"*บึงกาฬ*"),COUNTIF(B21,"*พังงา*"),COUNTIF(B21,"*ระนอง*"),COUNTIF(B21,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM21">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>2925773</v>
       </c>
-    </row>
-    <row r="22" spans="1:39">
+      <c r="AN21">
+        <v>9850</v>
+      </c>
+    </row>
+    <row r="22" spans="1:40">
       <c r="A22" t="s">
         <v>57</v>
       </c>
@@ -6217,16 +6263,18 @@
         <v>0</v>
       </c>
       <c r="AL22">
-        <f>IF(OR(COUNTIF(B22,"*กระบี่*"),COUNTIF(B22,"*จันทบุรี*"),COUNTIF(B22,"*ชุมพร*"),COUNTIF(B22,"*เชียงราย*"),COUNTIF(B22,"*ตรัง*"),COUNTIF(B22,"*นครนายก*"),COUNTIF(B22,"*ปราจีนบุรี*"),COUNTIF(B22,"*พัทลุง*"),COUNTIF(B22,"*ภูเก็ต*"),COUNTIF(B22,"*ยะลา*"),COUNTIF(B22,"*สกลนคร*"),COUNTIF(B22,"*สตูล*"),COUNTIF(B22,"*หนองคาย*"),COUNTIF(B22,"*สุราษฎร์ธานี*"),COUNTIF(B22,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B22,"*ตราด*"),COUNTIF(B22,"*นครพนม*"),COUNTIF(B22,"*นครศรีธรรมราช*"),COUNTIF(B22,"*นราธิวาส*"),COUNTIF(B22,"*บึงกาฬ*"),COUNTIF(B22,"*พังงา*"),COUNTIF(B22,"*ระนอง*"),COUNTIF(B22,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM22">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>14895309.58</v>
       </c>
-    </row>
-    <row r="23" spans="1:39">
+      <c r="AN22">
+        <v>9966.1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:40">
       <c r="A23" t="s">
         <v>57</v>
       </c>
@@ -6349,16 +6397,18 @@
         <v>0</v>
       </c>
       <c r="AL23">
-        <f>IF(OR(COUNTIF(B23,"*กระบี่*"),COUNTIF(B23,"*จันทบุรี*"),COUNTIF(B23,"*ชุมพร*"),COUNTIF(B23,"*เชียงราย*"),COUNTIF(B23,"*ตรัง*"),COUNTIF(B23,"*นครนายก*"),COUNTIF(B23,"*ปราจีนบุรี*"),COUNTIF(B23,"*พัทลุง*"),COUNTIF(B23,"*ภูเก็ต*"),COUNTIF(B23,"*ยะลา*"),COUNTIF(B23,"*สกลนคร*"),COUNTIF(B23,"*สตูล*"),COUNTIF(B23,"*หนองคาย*"),COUNTIF(B23,"*สุราษฎร์ธานี*"),COUNTIF(B23,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B23,"*ตราด*"),COUNTIF(B23,"*นครพนม*"),COUNTIF(B23,"*นครศรีธรรมราช*"),COUNTIF(B23,"*นราธิวาส*"),COUNTIF(B23,"*บึงกาฬ*"),COUNTIF(B23,"*พังงา*"),COUNTIF(B23,"*ระนอง*"),COUNTIF(B23,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM23">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>18362201</v>
       </c>
-    </row>
-    <row r="24" spans="1:39">
+      <c r="AN23">
+        <v>11938.45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:40">
       <c r="A24" t="s">
         <v>57</v>
       </c>
@@ -6481,16 +6531,18 @@
         <v>0</v>
       </c>
       <c r="AL24">
-        <f>IF(OR(COUNTIF(B24,"*กระบี่*"),COUNTIF(B24,"*จันทบุรี*"),COUNTIF(B24,"*ชุมพร*"),COUNTIF(B24,"*เชียงราย*"),COUNTIF(B24,"*ตรัง*"),COUNTIF(B24,"*นครนายก*"),COUNTIF(B24,"*ปราจีนบุรี*"),COUNTIF(B24,"*พัทลุง*"),COUNTIF(B24,"*ภูเก็ต*"),COUNTIF(B24,"*ยะลา*"),COUNTIF(B24,"*สกลนคร*"),COUNTIF(B24,"*สตูล*"),COUNTIF(B24,"*หนองคาย*"),COUNTIF(B24,"*สุราษฎร์ธานี*"),COUNTIF(B24,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B24,"*ตราด*"),COUNTIF(B24,"*นครพนม*"),COUNTIF(B24,"*นครศรีธรรมราช*"),COUNTIF(B24,"*นราธิวาส*"),COUNTIF(B24,"*บึงกาฬ*"),COUNTIF(B24,"*พังงา*"),COUNTIF(B24,"*ระนอง*"),COUNTIF(B24,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM24">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>23268968</v>
       </c>
-    </row>
-    <row r="25" spans="1:39">
+      <c r="AN24">
+        <v>9546.9110000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:40">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -6613,16 +6665,18 @@
         <v>0</v>
       </c>
       <c r="AL25">
-        <f>IF(OR(COUNTIF(B25,"*กระบี่*"),COUNTIF(B25,"*จันทบุรี*"),COUNTIF(B25,"*ชุมพร*"),COUNTIF(B25,"*เชียงราย*"),COUNTIF(B25,"*ตรัง*"),COUNTIF(B25,"*นครนายก*"),COUNTIF(B25,"*ปราจีนบุรี*"),COUNTIF(B25,"*พัทลุง*"),COUNTIF(B25,"*ภูเก็ต*"),COUNTIF(B25,"*ยะลา*"),COUNTIF(B25,"*สกลนคร*"),COUNTIF(B25,"*สตูล*"),COUNTIF(B25,"*หนองคาย*"),COUNTIF(B25,"*สุราษฎร์ธานี*"),COUNTIF(B25,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B25,"*ตราด*"),COUNTIF(B25,"*นครพนม*"),COUNTIF(B25,"*นครศรีธรรมราช*"),COUNTIF(B25,"*นราธิวาส*"),COUNTIF(B25,"*บึงกาฬ*"),COUNTIF(B25,"*พังงา*"),COUNTIF(B25,"*ระนอง*"),COUNTIF(B25,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM25">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>28246563.100000001</v>
       </c>
-    </row>
-    <row r="26" spans="1:39">
+      <c r="AN25">
+        <v>33899.955999999998</v>
+      </c>
+    </row>
+    <row r="26" spans="1:40">
       <c r="A26" t="s">
         <v>64</v>
       </c>
@@ -6745,16 +6799,18 @@
         <v>0</v>
       </c>
       <c r="AL26">
-        <f>IF(OR(COUNTIF(B26,"*กระบี่*"),COUNTIF(B26,"*จันทบุรี*"),COUNTIF(B26,"*ชุมพร*"),COUNTIF(B26,"*เชียงราย*"),COUNTIF(B26,"*ตรัง*"),COUNTIF(B26,"*นครนายก*"),COUNTIF(B26,"*ปราจีนบุรี*"),COUNTIF(B26,"*พัทลุง*"),COUNTIF(B26,"*ภูเก็ต*"),COUNTIF(B26,"*ยะลา*"),COUNTIF(B26,"*สกลนคร*"),COUNTIF(B26,"*สตูล*"),COUNTIF(B26,"*หนองคาย*"),COUNTIF(B26,"*สุราษฎร์ธานี*"),COUNTIF(B26,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B26,"*ตราด*"),COUNTIF(B26,"*นครพนม*"),COUNTIF(B26,"*นครศรีธรรมราช*"),COUNTIF(B26,"*นราธิวาส*"),COUNTIF(B26,"*บึงกาฬ*"),COUNTIF(B26,"*พังงา*"),COUNTIF(B26,"*ระนอง*"),COUNTIF(B26,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM26">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>17901066.350000001</v>
       </c>
-    </row>
-    <row r="27" spans="1:39">
+      <c r="AN26">
+        <v>28840.903999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:40">
       <c r="A27" t="s">
         <v>64</v>
       </c>
@@ -6877,16 +6933,18 @@
         <v>900000</v>
       </c>
       <c r="AL27">
-        <f>IF(OR(COUNTIF(B27,"*กระบี่*"),COUNTIF(B27,"*จันทบุรี*"),COUNTIF(B27,"*ชุมพร*"),COUNTIF(B27,"*เชียงราย*"),COUNTIF(B27,"*ตรัง*"),COUNTIF(B27,"*นครนายก*"),COUNTIF(B27,"*ปราจีนบุรี*"),COUNTIF(B27,"*พัทลุง*"),COUNTIF(B27,"*ภูเก็ต*"),COUNTIF(B27,"*ยะลา*"),COUNTIF(B27,"*สกลนคร*"),COUNTIF(B27,"*สตูล*"),COUNTIF(B27,"*หนองคาย*"),COUNTIF(B27,"*สุราษฎร์ธานี*"),COUNTIF(B27,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B27,"*ตราด*"),COUNTIF(B27,"*นครพนม*"),COUNTIF(B27,"*นครศรีธรรมราช*"),COUNTIF(B27,"*นราธิวาส*"),COUNTIF(B27,"*บึงกาฬ*"),COUNTIF(B27,"*พังงา*"),COUNTIF(B27,"*ระนอง*"),COUNTIF(B27,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AM27">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>22150559.68</v>
       </c>
-    </row>
-    <row r="28" spans="1:39">
+      <c r="AN27">
+        <v>11004.597</v>
+      </c>
+    </row>
+    <row r="28" spans="1:40">
       <c r="A28" t="s">
         <v>64</v>
       </c>
@@ -7009,16 +7067,18 @@
         <v>300000</v>
       </c>
       <c r="AL28">
-        <f>IF(OR(COUNTIF(B28,"*กระบี่*"),COUNTIF(B28,"*จันทบุรี*"),COUNTIF(B28,"*ชุมพร*"),COUNTIF(B28,"*เชียงราย*"),COUNTIF(B28,"*ตรัง*"),COUNTIF(B28,"*นครนายก*"),COUNTIF(B28,"*ปราจีนบุรี*"),COUNTIF(B28,"*พัทลุง*"),COUNTIF(B28,"*ภูเก็ต*"),COUNTIF(B28,"*ยะลา*"),COUNTIF(B28,"*สกลนคร*"),COUNTIF(B28,"*สตูล*"),COUNTIF(B28,"*หนองคาย*"),COUNTIF(B28,"*สุราษฎร์ธานี*"),COUNTIF(B28,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B28,"*ตราด*"),COUNTIF(B28,"*นครพนม*"),COUNTIF(B28,"*นครศรีธรรมราช*"),COUNTIF(B28,"*นราธิวาส*"),COUNTIF(B28,"*บึงกาฬ*"),COUNTIF(B28,"*พังงา*"),COUNTIF(B28,"*ระนอง*"),COUNTIF(B28,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM28">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>7450616</v>
       </c>
-    </row>
-    <row r="29" spans="1:39">
+      <c r="AN28">
+        <v>22085.925999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:40">
       <c r="A29" t="s">
         <v>64</v>
       </c>
@@ -7141,16 +7201,18 @@
         <v>900000</v>
       </c>
       <c r="AL29">
-        <f>IF(OR(COUNTIF(B29,"*กระบี่*"),COUNTIF(B29,"*จันทบุรี*"),COUNTIF(B29,"*ชุมพร*"),COUNTIF(B29,"*เชียงราย*"),COUNTIF(B29,"*ตรัง*"),COUNTIF(B29,"*นครนายก*"),COUNTIF(B29,"*ปราจีนบุรี*"),COUNTIF(B29,"*พัทลุง*"),COUNTIF(B29,"*ภูเก็ต*"),COUNTIF(B29,"*ยะลา*"),COUNTIF(B29,"*สกลนคร*"),COUNTIF(B29,"*สตูล*"),COUNTIF(B29,"*หนองคาย*"),COUNTIF(B29,"*สุราษฎร์ธานี*"),COUNTIF(B29,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B29,"*ตราด*"),COUNTIF(B29,"*นครพนม*"),COUNTIF(B29,"*นครศรีธรรมราช*"),COUNTIF(B29,"*นราธิวาส*"),COUNTIF(B29,"*บึงกาฬ*"),COUNTIF(B29,"*พังงา*"),COUNTIF(B29,"*ระนอง*"),COUNTIF(B29,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM29">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>94847495</v>
       </c>
-    </row>
-    <row r="30" spans="1:39">
+      <c r="AN29">
+        <v>37936.271999999997</v>
+      </c>
+    </row>
+    <row r="30" spans="1:40">
       <c r="A30" t="s">
         <v>64</v>
       </c>
@@ -7273,16 +7335,18 @@
         <v>0</v>
       </c>
       <c r="AL30">
-        <f>IF(OR(COUNTIF(B30,"*กระบี่*"),COUNTIF(B30,"*จันทบุรี*"),COUNTIF(B30,"*ชุมพร*"),COUNTIF(B30,"*เชียงราย*"),COUNTIF(B30,"*ตรัง*"),COUNTIF(B30,"*นครนายก*"),COUNTIF(B30,"*ปราจีนบุรี*"),COUNTIF(B30,"*พัทลุง*"),COUNTIF(B30,"*ภูเก็ต*"),COUNTIF(B30,"*ยะลา*"),COUNTIF(B30,"*สกลนคร*"),COUNTIF(B30,"*สตูล*"),COUNTIF(B30,"*หนองคาย*"),COUNTIF(B30,"*สุราษฎร์ธานี*"),COUNTIF(B30,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B30,"*ตราด*"),COUNTIF(B30,"*นครพนม*"),COUNTIF(B30,"*นครศรีธรรมราช*"),COUNTIF(B30,"*นราธิวาส*"),COUNTIF(B30,"*บึงกาฬ*"),COUNTIF(B30,"*พังงา*"),COUNTIF(B30,"*ระนอง*"),COUNTIF(B30,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM30">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>17975960.899999999</v>
       </c>
-    </row>
-    <row r="31" spans="1:39">
+      <c r="AN30">
+        <v>32991.050000000003</v>
+      </c>
+    </row>
+    <row r="31" spans="1:40">
       <c r="A31" t="s">
         <v>64</v>
       </c>
@@ -7405,16 +7469,18 @@
         <v>1800000</v>
       </c>
       <c r="AL31">
-        <f>IF(OR(COUNTIF(B31,"*กระบี่*"),COUNTIF(B31,"*จันทบุรี*"),COUNTIF(B31,"*ชุมพร*"),COUNTIF(B31,"*เชียงราย*"),COUNTIF(B31,"*ตรัง*"),COUNTIF(B31,"*นครนายก*"),COUNTIF(B31,"*ปราจีนบุรี*"),COUNTIF(B31,"*พัทลุง*"),COUNTIF(B31,"*ภูเก็ต*"),COUNTIF(B31,"*ยะลา*"),COUNTIF(B31,"*สกลนคร*"),COUNTIF(B31,"*สตูล*"),COUNTIF(B31,"*หนองคาย*"),COUNTIF(B31,"*สุราษฎร์ธานี*"),COUNTIF(B31,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B31,"*ตราด*"),COUNTIF(B31,"*นครพนม*"),COUNTIF(B31,"*นครศรีธรรมราช*"),COUNTIF(B31,"*นราธิวาส*"),COUNTIF(B31,"*บึงกาฬ*"),COUNTIF(B31,"*พังงา*"),COUNTIF(B31,"*ระนอง*"),COUNTIF(B31,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM31">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>26396681.800000001</v>
       </c>
-    </row>
-    <row r="32" spans="1:39">
+      <c r="AN31">
+        <v>34391.175000000003</v>
+      </c>
+    </row>
+    <row r="32" spans="1:40">
       <c r="A32" t="s">
         <v>64</v>
       </c>
@@ -7537,16 +7603,18 @@
         <v>0</v>
       </c>
       <c r="AL32">
-        <f>IF(OR(COUNTIF(B32,"*กระบี่*"),COUNTIF(B32,"*จันทบุรี*"),COUNTIF(B32,"*ชุมพร*"),COUNTIF(B32,"*เชียงราย*"),COUNTIF(B32,"*ตรัง*"),COUNTIF(B32,"*นครนายก*"),COUNTIF(B32,"*ปราจีนบุรี*"),COUNTIF(B32,"*พัทลุง*"),COUNTIF(B32,"*ภูเก็ต*"),COUNTIF(B32,"*ยะลา*"),COUNTIF(B32,"*สกลนคร*"),COUNTIF(B32,"*สตูล*"),COUNTIF(B32,"*หนองคาย*"),COUNTIF(B32,"*สุราษฎร์ธานี*"),COUNTIF(B32,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B32,"*ตราด*"),COUNTIF(B32,"*นครพนม*"),COUNTIF(B32,"*นครศรีธรรมราช*"),COUNTIF(B32,"*นราธิวาส*"),COUNTIF(B32,"*บึงกาฬ*"),COUNTIF(B32,"*พังงา*"),COUNTIF(B32,"*ระนอง*"),COUNTIF(B32,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM32">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>39174819.990000002</v>
       </c>
-    </row>
-    <row r="33" spans="1:39">
+      <c r="AN32">
+        <v>41046.665999999997</v>
+      </c>
+    </row>
+    <row r="33" spans="1:40">
       <c r="A33" t="s">
         <v>73</v>
       </c>
@@ -7669,16 +7737,18 @@
         <v>300000</v>
       </c>
       <c r="AL33">
-        <f>IF(OR(COUNTIF(B33,"*กระบี่*"),COUNTIF(B33,"*จันทบุรี*"),COUNTIF(B33,"*ชุมพร*"),COUNTIF(B33,"*เชียงราย*"),COUNTIF(B33,"*ตรัง*"),COUNTIF(B33,"*นครนายก*"),COUNTIF(B33,"*ปราจีนบุรี*"),COUNTIF(B33,"*พัทลุง*"),COUNTIF(B33,"*ภูเก็ต*"),COUNTIF(B33,"*ยะลา*"),COUNTIF(B33,"*สกลนคร*"),COUNTIF(B33,"*สตูล*"),COUNTIF(B33,"*หนองคาย*"),COUNTIF(B33,"*สุราษฎร์ธานี*"),COUNTIF(B33,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B33,"*ตราด*"),COUNTIF(B33,"*นครพนม*"),COUNTIF(B33,"*นครศรีธรรมราช*"),COUNTIF(B33,"*นราธิวาส*"),COUNTIF(B33,"*บึงกาฬ*"),COUNTIF(B33,"*พังงา*"),COUNTIF(B33,"*ระนอง*"),COUNTIF(B33,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AM33">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>44418991.719999999</v>
       </c>
-    </row>
-    <row r="34" spans="1:39">
+      <c r="AN33">
+        <v>20978.356</v>
+      </c>
+    </row>
+    <row r="34" spans="1:40">
       <c r="A34" t="s">
         <v>73</v>
       </c>
@@ -7801,7 +7871,7 @@
         <v>600000</v>
       </c>
       <c r="AL34">
-        <f>IF(OR(COUNTIF(B34,"*กระบี่*"),COUNTIF(B34,"*จันทบุรี*"),COUNTIF(B34,"*ชุมพร*"),COUNTIF(B34,"*เชียงราย*"),COUNTIF(B34,"*ตรัง*"),COUNTIF(B34,"*นครนายก*"),COUNTIF(B34,"*ปราจีนบุรี*"),COUNTIF(B34,"*พัทลุง*"),COUNTIF(B34,"*ภูเก็ต*"),COUNTIF(B34,"*ยะลา*"),COUNTIF(B34,"*สกลนคร*"),COUNTIF(B34,"*สตูล*"),COUNTIF(B34,"*หนองคาย*"),COUNTIF(B34,"*สุราษฎร์ธานี*"),COUNTIF(B34,"*ปัตตานี*")),2,
+        <f t="shared" ref="AL34:AL65" si="1">IF(OR(COUNTIF(B34,"*กระบี่*"),COUNTIF(B34,"*จันทบุรี*"),COUNTIF(B34,"*ชุมพร*"),COUNTIF(B34,"*เชียงราย*"),COUNTIF(B34,"*ตรัง*"),COUNTIF(B34,"*นครนายก*"),COUNTIF(B34,"*ปราจีนบุรี*"),COUNTIF(B34,"*พัทลุง*"),COUNTIF(B34,"*ภูเก็ต*"),COUNTIF(B34,"*ยะลา*"),COUNTIF(B34,"*สกลนคร*"),COUNTIF(B34,"*สตูล*"),COUNTIF(B34,"*หนองคาย*"),COUNTIF(B34,"*สุราษฎร์ธานี*"),COUNTIF(B34,"*ปัตตานี*")),2,
 IF(OR(COUNTIF(B34,"*ตราด*"),COUNTIF(B34,"*นครพนม*"),COUNTIF(B34,"*นครศรีธรรมราช*"),COUNTIF(B34,"*นราธิวาส*"),COUNTIF(B34,"*บึงกาฬ*"),COUNTIF(B34,"*พังงา*"),COUNTIF(B34,"*ระนอง*"),COUNTIF(B34,"*สงขลา*")),4,0))</f>
         <v>0</v>
       </c>
@@ -7809,8 +7879,11 @@
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>38774837.789999999</v>
       </c>
-    </row>
-    <row r="35" spans="1:39">
+      <c r="AN34">
+        <v>7966.9279999999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:40">
       <c r="A35" t="s">
         <v>73</v>
       </c>
@@ -7933,16 +8006,18 @@
         <v>600000</v>
       </c>
       <c r="AL35">
-        <f>IF(OR(COUNTIF(B35,"*กระบี่*"),COUNTIF(B35,"*จันทบุรี*"),COUNTIF(B35,"*ชุมพร*"),COUNTIF(B35,"*เชียงราย*"),COUNTIF(B35,"*ตรัง*"),COUNTIF(B35,"*นครนายก*"),COUNTIF(B35,"*ปราจีนบุรี*"),COUNTIF(B35,"*พัทลุง*"),COUNTIF(B35,"*ภูเก็ต*"),COUNTIF(B35,"*ยะลา*"),COUNTIF(B35,"*สกลนคร*"),COUNTIF(B35,"*สตูล*"),COUNTIF(B35,"*หนองคาย*"),COUNTIF(B35,"*สุราษฎร์ธานี*"),COUNTIF(B35,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B35,"*ตราด*"),COUNTIF(B35,"*นครพนม*"),COUNTIF(B35,"*นครศรีธรรมราช*"),COUNTIF(B35,"*นราธิวาส*"),COUNTIF(B35,"*บึงกาฬ*"),COUNTIF(B35,"*พังงา*"),COUNTIF(B35,"*ระนอง*"),COUNTIF(B35,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="AM35">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>24685294.829999998</v>
       </c>
-    </row>
-    <row r="36" spans="1:39">
+      <c r="AN35">
+        <v>5399</v>
+      </c>
+    </row>
+    <row r="36" spans="1:40">
       <c r="A36" t="s">
         <v>73</v>
       </c>
@@ -8065,16 +8140,18 @@
         <v>0</v>
       </c>
       <c r="AL36">
-        <f>IF(OR(COUNTIF(B36,"*กระบี่*"),COUNTIF(B36,"*จันทบุรี*"),COUNTIF(B36,"*ชุมพร*"),COUNTIF(B36,"*เชียงราย*"),COUNTIF(B36,"*ตรัง*"),COUNTIF(B36,"*นครนายก*"),COUNTIF(B36,"*ปราจีนบุรี*"),COUNTIF(B36,"*พัทลุง*"),COUNTIF(B36,"*ภูเก็ต*"),COUNTIF(B36,"*ยะลา*"),COUNTIF(B36,"*สกลนคร*"),COUNTIF(B36,"*สตูล*"),COUNTIF(B36,"*หนองคาย*"),COUNTIF(B36,"*สุราษฎร์ธานี*"),COUNTIF(B36,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B36,"*ตราด*"),COUNTIF(B36,"*นครพนม*"),COUNTIF(B36,"*นครศรีธรรมราช*"),COUNTIF(B36,"*นราธิวาส*"),COUNTIF(B36,"*บึงกาฬ*"),COUNTIF(B36,"*พังงา*"),COUNTIF(B36,"*ระนอง*"),COUNTIF(B36,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="AM36">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>18951930.5</v>
       </c>
-    </row>
-    <row r="37" spans="1:39">
+      <c r="AN36">
+        <v>6707</v>
+      </c>
+    </row>
+    <row r="37" spans="1:40">
       <c r="A37" t="s">
         <v>73</v>
       </c>
@@ -8197,16 +8274,18 @@
         <v>0</v>
       </c>
       <c r="AL37">
-        <f>IF(OR(COUNTIF(B37,"*กระบี่*"),COUNTIF(B37,"*จันทบุรี*"),COUNTIF(B37,"*ชุมพร*"),COUNTIF(B37,"*เชียงราย*"),COUNTIF(B37,"*ตรัง*"),COUNTIF(B37,"*นครนายก*"),COUNTIF(B37,"*ปราจีนบุรี*"),COUNTIF(B37,"*พัทลุง*"),COUNTIF(B37,"*ภูเก็ต*"),COUNTIF(B37,"*ยะลา*"),COUNTIF(B37,"*สกลนคร*"),COUNTIF(B37,"*สตูล*"),COUNTIF(B37,"*หนองคาย*"),COUNTIF(B37,"*สุราษฎร์ธานี*"),COUNTIF(B37,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B37,"*ตราด*"),COUNTIF(B37,"*นครพนม*"),COUNTIF(B37,"*นครศรีธรรมราช*"),COUNTIF(B37,"*นราธิวาส*"),COUNTIF(B37,"*บึงกาฬ*"),COUNTIF(B37,"*พังงา*"),COUNTIF(B37,"*ระนอง*"),COUNTIF(B37,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM37">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>3241211.73</v>
       </c>
-    </row>
-    <row r="38" spans="1:39">
+      <c r="AN37">
+        <v>8861.7000000000007</v>
+      </c>
+    </row>
+    <row r="38" spans="1:40">
       <c r="A38" t="s">
         <v>73</v>
       </c>
@@ -8329,16 +8408,18 @@
         <v>0</v>
       </c>
       <c r="AL38">
-        <f>IF(OR(COUNTIF(B38,"*กระบี่*"),COUNTIF(B38,"*จันทบุรี*"),COUNTIF(B38,"*ชุมพร*"),COUNTIF(B38,"*เชียงราย*"),COUNTIF(B38,"*ตรัง*"),COUNTIF(B38,"*นครนายก*"),COUNTIF(B38,"*ปราจีนบุรี*"),COUNTIF(B38,"*พัทลุง*"),COUNTIF(B38,"*ภูเก็ต*"),COUNTIF(B38,"*ยะลา*"),COUNTIF(B38,"*สกลนคร*"),COUNTIF(B38,"*สตูล*"),COUNTIF(B38,"*หนองคาย*"),COUNTIF(B38,"*สุราษฎร์ธานี*"),COUNTIF(B38,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B38,"*ตราด*"),COUNTIF(B38,"*นครพนม*"),COUNTIF(B38,"*นครศรีธรรมราช*"),COUNTIF(B38,"*นราธิวาส*"),COUNTIF(B38,"*บึงกาฬ*"),COUNTIF(B38,"*พังงา*"),COUNTIF(B38,"*ระนอง*"),COUNTIF(B38,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM38">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>21623707.629999999</v>
       </c>
-    </row>
-    <row r="39" spans="1:39">
+      <c r="AN38">
+        <v>18811.3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:40">
       <c r="A39" t="s">
         <v>80</v>
       </c>
@@ -8461,16 +8542,18 @@
         <v>600000</v>
       </c>
       <c r="AL39">
-        <f>IF(OR(COUNTIF(B39,"*กระบี่*"),COUNTIF(B39,"*จันทบุรี*"),COUNTIF(B39,"*ชุมพร*"),COUNTIF(B39,"*เชียงราย*"),COUNTIF(B39,"*ตรัง*"),COUNTIF(B39,"*นครนายก*"),COUNTIF(B39,"*ปราจีนบุรี*"),COUNTIF(B39,"*พัทลุง*"),COUNTIF(B39,"*ภูเก็ต*"),COUNTIF(B39,"*ยะลา*"),COUNTIF(B39,"*สกลนคร*"),COUNTIF(B39,"*สตูล*"),COUNTIF(B39,"*หนองคาย*"),COUNTIF(B39,"*สุราษฎร์ธานี*"),COUNTIF(B39,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B39,"*ตราด*"),COUNTIF(B39,"*นครพนม*"),COUNTIF(B39,"*นครศรีธรรมราช*"),COUNTIF(B39,"*นราธิวาส*"),COUNTIF(B39,"*บึงกาฬ*"),COUNTIF(B39,"*พังงา*"),COUNTIF(B39,"*ระนอง*"),COUNTIF(B39,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM39">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>24056530.640000001</v>
       </c>
-    </row>
-    <row r="40" spans="1:39">
+      <c r="AN39">
+        <v>4541</v>
+      </c>
+    </row>
+    <row r="40" spans="1:40">
       <c r="A40" t="s">
         <v>80</v>
       </c>
@@ -8593,16 +8676,18 @@
         <v>600000</v>
       </c>
       <c r="AL40">
-        <f>IF(OR(COUNTIF(B40,"*กระบี่*"),COUNTIF(B40,"*จันทบุรี*"),COUNTIF(B40,"*ชุมพร*"),COUNTIF(B40,"*เชียงราย*"),COUNTIF(B40,"*ตรัง*"),COUNTIF(B40,"*นครนายก*"),COUNTIF(B40,"*ปราจีนบุรี*"),COUNTIF(B40,"*พัทลุง*"),COUNTIF(B40,"*ภูเก็ต*"),COUNTIF(B40,"*ยะลา*"),COUNTIF(B40,"*สกลนคร*"),COUNTIF(B40,"*สตูล*"),COUNTIF(B40,"*หนองคาย*"),COUNTIF(B40,"*สุราษฎร์ธานี*"),COUNTIF(B40,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B40,"*ตราด*"),COUNTIF(B40,"*นครพนม*"),COUNTIF(B40,"*นครศรีธรรมราช*"),COUNTIF(B40,"*นราธิวาส*"),COUNTIF(B40,"*บึงกาฬ*"),COUNTIF(B40,"*พังงา*"),COUNTIF(B40,"*ระนอง*"),COUNTIF(B40,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM40">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>15892650.960000001</v>
       </c>
-    </row>
-    <row r="41" spans="1:39">
+      <c r="AN40">
+        <v>24167.035</v>
+      </c>
+    </row>
+    <row r="41" spans="1:40">
       <c r="A41" t="s">
         <v>80</v>
       </c>
@@ -8725,16 +8810,18 @@
         <v>600000</v>
       </c>
       <c r="AL41">
-        <f>IF(OR(COUNTIF(B41,"*กระบี่*"),COUNTIF(B41,"*จันทบุรี*"),COUNTIF(B41,"*ชุมพร*"),COUNTIF(B41,"*เชียงราย*"),COUNTIF(B41,"*ตรัง*"),COUNTIF(B41,"*นครนายก*"),COUNTIF(B41,"*ปราจีนบุรี*"),COUNTIF(B41,"*พัทลุง*"),COUNTIF(B41,"*ภูเก็ต*"),COUNTIF(B41,"*ยะลา*"),COUNTIF(B41,"*สกลนคร*"),COUNTIF(B41,"*สตูล*"),COUNTIF(B41,"*หนองคาย*"),COUNTIF(B41,"*สุราษฎร์ธานี*"),COUNTIF(B41,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B41,"*ตราด*"),COUNTIF(B41,"*นครพนม*"),COUNTIF(B41,"*นครศรีธรรมราช*"),COUNTIF(B41,"*นราธิวาส*"),COUNTIF(B41,"*บึงกาฬ*"),COUNTIF(B41,"*พังงา*"),COUNTIF(B41,"*ระนอง*"),COUNTIF(B41,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM41">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>10931073</v>
       </c>
-    </row>
-    <row r="42" spans="1:39">
+      <c r="AN41">
+        <v>4437.1000000000004</v>
+      </c>
+    </row>
+    <row r="42" spans="1:40">
       <c r="A42" t="s">
         <v>80</v>
       </c>
@@ -8851,16 +8938,18 @@
         <v>0</v>
       </c>
       <c r="AL42">
-        <f>IF(OR(COUNTIF(B42,"*กระบี่*"),COUNTIF(B42,"*จันทบุรี*"),COUNTIF(B42,"*ชุมพร*"),COUNTIF(B42,"*เชียงราย*"),COUNTIF(B42,"*ตรัง*"),COUNTIF(B42,"*นครนายก*"),COUNTIF(B42,"*ปราจีนบุรี*"),COUNTIF(B42,"*พัทลุง*"),COUNTIF(B42,"*ภูเก็ต*"),COUNTIF(B42,"*ยะลา*"),COUNTIF(B42,"*สกลนคร*"),COUNTIF(B42,"*สตูล*"),COUNTIF(B42,"*หนองคาย*"),COUNTIF(B42,"*สุราษฎร์ธานี*"),COUNTIF(B42,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B42,"*ตราด*"),COUNTIF(B42,"*นครพนม*"),COUNTIF(B42,"*นครศรีธรรมราช*"),COUNTIF(B42,"*นราธิวาส*"),COUNTIF(B42,"*บึงกาฬ*"),COUNTIF(B42,"*พังงา*"),COUNTIF(B42,"*ระนอง*"),COUNTIF(B42,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM42">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>21907259</v>
       </c>
-    </row>
-    <row r="43" spans="1:39">
+      <c r="AN42">
+        <v>5163</v>
+      </c>
+    </row>
+    <row r="43" spans="1:40">
       <c r="A43" t="s">
         <v>80</v>
       </c>
@@ -8983,16 +9072,18 @@
         <v>900000</v>
       </c>
       <c r="AL43">
-        <f>IF(OR(COUNTIF(B43,"*กระบี่*"),COUNTIF(B43,"*จันทบุรี*"),COUNTIF(B43,"*ชุมพร*"),COUNTIF(B43,"*เชียงราย*"),COUNTIF(B43,"*ตรัง*"),COUNTIF(B43,"*นครนายก*"),COUNTIF(B43,"*ปราจีนบุรี*"),COUNTIF(B43,"*พัทลุง*"),COUNTIF(B43,"*ภูเก็ต*"),COUNTIF(B43,"*ยะลา*"),COUNTIF(B43,"*สกลนคร*"),COUNTIF(B43,"*สตูล*"),COUNTIF(B43,"*หนองคาย*"),COUNTIF(B43,"*สุราษฎร์ธานี*"),COUNTIF(B43,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B43,"*ตราด*"),COUNTIF(B43,"*นครพนม*"),COUNTIF(B43,"*นครศรีธรรมราช*"),COUNTIF(B43,"*นราธิวาส*"),COUNTIF(B43,"*บึงกาฬ*"),COUNTIF(B43,"*พังงา*"),COUNTIF(B43,"*ระนอง*"),COUNTIF(B43,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM43">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>23134918.710000001</v>
       </c>
-    </row>
-    <row r="44" spans="1:39">
+      <c r="AN43">
+        <v>12625.6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:40">
       <c r="A44" t="s">
         <v>80</v>
       </c>
@@ -9115,16 +9206,18 @@
         <v>300000</v>
       </c>
       <c r="AL44">
-        <f>IF(OR(COUNTIF(B44,"*กระบี่*"),COUNTIF(B44,"*จันทบุรี*"),COUNTIF(B44,"*ชุมพร*"),COUNTIF(B44,"*เชียงราย*"),COUNTIF(B44,"*ตรัง*"),COUNTIF(B44,"*นครนายก*"),COUNTIF(B44,"*ปราจีนบุรี*"),COUNTIF(B44,"*พัทลุง*"),COUNTIF(B44,"*ภูเก็ต*"),COUNTIF(B44,"*ยะลา*"),COUNTIF(B44,"*สกลนคร*"),COUNTIF(B44,"*สตูล*"),COUNTIF(B44,"*หนองคาย*"),COUNTIF(B44,"*สุราษฎร์ธานี*"),COUNTIF(B44,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B44,"*ตราด*"),COUNTIF(B44,"*นครพนม*"),COUNTIF(B44,"*นครศรีธรรมราช*"),COUNTIF(B44,"*นราธิวาส*"),COUNTIF(B44,"*บึงกาฬ*"),COUNTIF(B44,"*พังงา*"),COUNTIF(B44,"*ระนอง*"),COUNTIF(B44,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM44">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>44864899.299999997</v>
       </c>
-    </row>
-    <row r="45" spans="1:39">
+      <c r="AN44">
+        <v>3871</v>
+      </c>
+    </row>
+    <row r="45" spans="1:40">
       <c r="A45" t="s">
         <v>87</v>
       </c>
@@ -9247,16 +9340,18 @@
         <v>0</v>
       </c>
       <c r="AL45">
-        <f>IF(OR(COUNTIF(B45,"*กระบี่*"),COUNTIF(B45,"*จันทบุรี*"),COUNTIF(B45,"*ชุมพร*"),COUNTIF(B45,"*เชียงราย*"),COUNTIF(B45,"*ตรัง*"),COUNTIF(B45,"*นครนายก*"),COUNTIF(B45,"*ปราจีนบุรี*"),COUNTIF(B45,"*พัทลุง*"),COUNTIF(B45,"*ภูเก็ต*"),COUNTIF(B45,"*ยะลา*"),COUNTIF(B45,"*สกลนคร*"),COUNTIF(B45,"*สตูล*"),COUNTIF(B45,"*หนองคาย*"),COUNTIF(B45,"*สุราษฎร์ธานี*"),COUNTIF(B45,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B45,"*ตราด*"),COUNTIF(B45,"*นครพนม*"),COUNTIF(B45,"*นครศรีธรรมราช*"),COUNTIF(B45,"*นราธิวาส*"),COUNTIF(B45,"*บึงกาฬ*"),COUNTIF(B45,"*พังงา*"),COUNTIF(B45,"*ระนอง*"),COUNTIF(B45,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM45">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>9436328.3399999999</v>
       </c>
-    </row>
-    <row r="46" spans="1:39">
+      <c r="AN45">
+        <v>21833</v>
+      </c>
+    </row>
+    <row r="46" spans="1:40">
       <c r="A46" t="s">
         <v>87</v>
       </c>
@@ -9379,16 +9474,18 @@
         <v>0</v>
       </c>
       <c r="AL46">
-        <f>IF(OR(COUNTIF(B46,"*กระบี่*"),COUNTIF(B46,"*จันทบุรี*"),COUNTIF(B46,"*ชุมพร*"),COUNTIF(B46,"*เชียงราย*"),COUNTIF(B46,"*ตรัง*"),COUNTIF(B46,"*นครนายก*"),COUNTIF(B46,"*ปราจีนบุรี*"),COUNTIF(B46,"*พัทลุง*"),COUNTIF(B46,"*ภูเก็ต*"),COUNTIF(B46,"*ยะลา*"),COUNTIF(B46,"*สกลนคร*"),COUNTIF(B46,"*สตูล*"),COUNTIF(B46,"*หนองคาย*"),COUNTIF(B46,"*สุราษฎร์ธานี*"),COUNTIF(B46,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B46,"*ตราด*"),COUNTIF(B46,"*นครพนม*"),COUNTIF(B46,"*นครศรีธรรมราช*"),COUNTIF(B46,"*นราธิวาส*"),COUNTIF(B46,"*บึงกาฬ*"),COUNTIF(B46,"*พังงา*"),COUNTIF(B46,"*ระนอง*"),COUNTIF(B46,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM46">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>13052440.210000001</v>
       </c>
-    </row>
-    <row r="47" spans="1:39">
+      <c r="AN46">
+        <v>4937</v>
+      </c>
+    </row>
+    <row r="47" spans="1:40">
       <c r="A47" t="s">
         <v>87</v>
       </c>
@@ -9511,16 +9608,18 @@
         <v>300000</v>
       </c>
       <c r="AL47">
-        <f>IF(OR(COUNTIF(B47,"*กระบี่*"),COUNTIF(B47,"*จันทบุรี*"),COUNTIF(B47,"*ชุมพร*"),COUNTIF(B47,"*เชียงราย*"),COUNTIF(B47,"*ตรัง*"),COUNTIF(B47,"*นครนายก*"),COUNTIF(B47,"*ปราจีนบุรี*"),COUNTIF(B47,"*พัทลุง*"),COUNTIF(B47,"*ภูเก็ต*"),COUNTIF(B47,"*ยะลา*"),COUNTIF(B47,"*สกลนคร*"),COUNTIF(B47,"*สตูล*"),COUNTIF(B47,"*หนองคาย*"),COUNTIF(B47,"*สุราษฎร์ธานี*"),COUNTIF(B47,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B47,"*ตราด*"),COUNTIF(B47,"*นครพนม*"),COUNTIF(B47,"*นครศรีธรรมราช*"),COUNTIF(B47,"*นราธิวาส*"),COUNTIF(B47,"*บึงกาฬ*"),COUNTIF(B47,"*พังงา*"),COUNTIF(B47,"*ระนอง*"),COUNTIF(B47,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM47">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>22849661</v>
       </c>
-    </row>
-    <row r="48" spans="1:39">
+      <c r="AN47">
+        <v>5370.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:40">
       <c r="A48" t="s">
         <v>87</v>
       </c>
@@ -9643,20 +9742,22 @@
         <v>300000</v>
       </c>
       <c r="AL48">
-        <f>IF(OR(COUNTIF(B48,"*กระบี่*"),COUNTIF(B48,"*จันทบุรี*"),COUNTIF(B48,"*ชุมพร*"),COUNTIF(B48,"*เชียงราย*"),COUNTIF(B48,"*ตรัง*"),COUNTIF(B48,"*นครนายก*"),COUNTIF(B48,"*ปราจีนบุรี*"),COUNTIF(B48,"*พัทลุง*"),COUNTIF(B48,"*ภูเก็ต*"),COUNTIF(B48,"*ยะลา*"),COUNTIF(B48,"*สกลนคร*"),COUNTIF(B48,"*สตูล*"),COUNTIF(B48,"*หนองคาย*"),COUNTIF(B48,"*สุราษฎร์ธานี*"),COUNTIF(B48,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B48,"*ตราด*"),COUNTIF(B48,"*นครพนม*"),COUNTIF(B48,"*นครศรีธรรมราช*"),COUNTIF(B48,"*นราธิวาส*"),COUNTIF(B48,"*บึงกาฬ*"),COUNTIF(B48,"*พังงา*"),COUNTIF(B48,"*ระนอง*"),COUNTIF(B48,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM48">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>25981167</v>
       </c>
-    </row>
-    <row r="49" spans="1:39">
+      <c r="AN48">
+        <v>5696</v>
+      </c>
+    </row>
+    <row r="49" spans="1:40">
       <c r="A49" t="s">
         <v>87</v>
       </c>
-      <c r="B49" s="82" t="s">
+      <c r="B49" t="s">
         <v>92</v>
       </c>
       <c r="C49" s="39">
@@ -9775,16 +9876,18 @@
         <v>0</v>
       </c>
       <c r="AL49">
-        <f>IF(OR(COUNTIF(B49,"*กระบี่*"),COUNTIF(B49,"*จันทบุรี*"),COUNTIF(B49,"*ชุมพร*"),COUNTIF(B49,"*เชียงราย*"),COUNTIF(B49,"*ตรัง*"),COUNTIF(B49,"*นครนายก*"),COUNTIF(B49,"*ปราจีนบุรี*"),COUNTIF(B49,"*พัทลุง*"),COUNTIF(B49,"*ภูเก็ต*"),COUNTIF(B49,"*ยะลา*"),COUNTIF(B49,"*สกลนคร*"),COUNTIF(B49,"*สตูล*"),COUNTIF(B49,"*หนองคาย*"),COUNTIF(B49,"*สุราษฎร์ธานี*"),COUNTIF(B49,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B49,"*ตราด*"),COUNTIF(B49,"*นครพนม*"),COUNTIF(B49,"*นครศรีธรรมราช*"),COUNTIF(B49,"*นราธิวาส*"),COUNTIF(B49,"*บึงกาฬ*"),COUNTIF(B49,"*พังงา*"),COUNTIF(B49,"*ระนอง*"),COUNTIF(B49,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM49">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>8096662</v>
       </c>
-    </row>
-    <row r="50" spans="1:39">
+      <c r="AN49">
+        <v>3668.85</v>
+      </c>
+    </row>
+    <row r="50" spans="1:40">
       <c r="A50" t="s">
         <v>87</v>
       </c>
@@ -9907,16 +10010,18 @@
         <v>0</v>
       </c>
       <c r="AL50">
-        <f>IF(OR(COUNTIF(B50,"*กระบี่*"),COUNTIF(B50,"*จันทบุรี*"),COUNTIF(B50,"*ชุมพร*"),COUNTIF(B50,"*เชียงราย*"),COUNTIF(B50,"*ตรัง*"),COUNTIF(B50,"*นครนายก*"),COUNTIF(B50,"*ปราจีนบุรี*"),COUNTIF(B50,"*พัทลุง*"),COUNTIF(B50,"*ภูเก็ต*"),COUNTIF(B50,"*ยะลา*"),COUNTIF(B50,"*สกลนคร*"),COUNTIF(B50,"*สตูล*"),COUNTIF(B50,"*หนองคาย*"),COUNTIF(B50,"*สุราษฎร์ธานี*"),COUNTIF(B50,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B50,"*ตราด*"),COUNTIF(B50,"*นครพนม*"),COUNTIF(B50,"*นครศรีธรรมราช*"),COUNTIF(B50,"*นราธิวาส*"),COUNTIF(B50,"*บึงกาฬ*"),COUNTIF(B50,"*พังงา*"),COUNTIF(B50,"*ระนอง*"),COUNTIF(B50,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM50">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>21647068.02</v>
       </c>
-    </row>
-    <row r="51" spans="1:39">
+      <c r="AN50">
+        <v>11842</v>
+      </c>
+    </row>
+    <row r="51" spans="1:40">
       <c r="A51" t="s">
         <v>94</v>
       </c>
@@ -10039,16 +10144,18 @@
         <v>300000</v>
       </c>
       <c r="AL51">
-        <f>IF(OR(COUNTIF(B51,"*กระบี่*"),COUNTIF(B51,"*จันทบุรี*"),COUNTIF(B51,"*ชุมพร*"),COUNTIF(B51,"*เชียงราย*"),COUNTIF(B51,"*ตรัง*"),COUNTIF(B51,"*นครนายก*"),COUNTIF(B51,"*ปราจีนบุรี*"),COUNTIF(B51,"*พัทลุง*"),COUNTIF(B51,"*ภูเก็ต*"),COUNTIF(B51,"*ยะลา*"),COUNTIF(B51,"*สกลนคร*"),COUNTIF(B51,"*สตูล*"),COUNTIF(B51,"*หนองคาย*"),COUNTIF(B51,"*สุราษฎร์ธานี*"),COUNTIF(B51,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B51,"*ตราด*"),COUNTIF(B51,"*นครพนม*"),COUNTIF(B51,"*นครศรีธรรมราช*"),COUNTIF(B51,"*นราธิวาส*"),COUNTIF(B51,"*บึงกาฬ*"),COUNTIF(B51,"*พังงา*"),COUNTIF(B51,"*ระนอง*"),COUNTIF(B51,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM51">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>25873713.629999999</v>
       </c>
-    </row>
-    <row r="52" spans="1:39">
+      <c r="AN51">
+        <v>10628</v>
+      </c>
+    </row>
+    <row r="52" spans="1:40">
       <c r="A52" t="s">
         <v>96</v>
       </c>
@@ -10171,16 +10278,18 @@
         <v>600000</v>
       </c>
       <c r="AL52">
-        <f>IF(OR(COUNTIF(B52,"*กระบี่*"),COUNTIF(B52,"*จันทบุรี*"),COUNTIF(B52,"*ชุมพร*"),COUNTIF(B52,"*เชียงราย*"),COUNTIF(B52,"*ตรัง*"),COUNTIF(B52,"*นครนายก*"),COUNTIF(B52,"*ปราจีนบุรี*"),COUNTIF(B52,"*พัทลุง*"),COUNTIF(B52,"*ภูเก็ต*"),COUNTIF(B52,"*ยะลา*"),COUNTIF(B52,"*สกลนคร*"),COUNTIF(B52,"*สตูล*"),COUNTIF(B52,"*หนองคาย*"),COUNTIF(B52,"*สุราษฎร์ธานี*"),COUNTIF(B52,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B52,"*ตราด*"),COUNTIF(B52,"*นครพนม*"),COUNTIF(B52,"*นครศรีธรรมราช*"),COUNTIF(B52,"*นราธิวาส*"),COUNTIF(B52,"*บึงกาฬ*"),COUNTIF(B52,"*พังงา*"),COUNTIF(B52,"*ระนอง*"),COUNTIF(B52,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM52">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>16304171.380000001</v>
       </c>
-    </row>
-    <row r="53" spans="1:39">
+      <c r="AN52">
+        <v>8321.6</v>
+      </c>
+    </row>
+    <row r="53" spans="1:40">
       <c r="A53" t="s">
         <v>96</v>
       </c>
@@ -10303,16 +10412,18 @@
         <v>300000</v>
       </c>
       <c r="AL53">
-        <f>IF(OR(COUNTIF(B53,"*กระบี่*"),COUNTIF(B53,"*จันทบุรี*"),COUNTIF(B53,"*ชุมพร*"),COUNTIF(B53,"*เชียงราย*"),COUNTIF(B53,"*ตรัง*"),COUNTIF(B53,"*นครนายก*"),COUNTIF(B53,"*ปราจีนบุรี*"),COUNTIF(B53,"*พัทลุง*"),COUNTIF(B53,"*ภูเก็ต*"),COUNTIF(B53,"*ยะลา*"),COUNTIF(B53,"*สกลนคร*"),COUNTIF(B53,"*สตูล*"),COUNTIF(B53,"*หนองคาย*"),COUNTIF(B53,"*สุราษฎร์ธานี*"),COUNTIF(B53,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B53,"*ตราด*"),COUNTIF(B53,"*นครพนม*"),COUNTIF(B53,"*นครศรีธรรมราช*"),COUNTIF(B53,"*นราธิวาส*"),COUNTIF(B53,"*บึงกาฬ*"),COUNTIF(B53,"*พังงา*"),COUNTIF(B53,"*ระนอง*"),COUNTIF(B53,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM53">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>21915969</v>
       </c>
-    </row>
-    <row r="54" spans="1:39">
+      <c r="AN53">
+        <v>8524.9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:40">
       <c r="A54" t="s">
         <v>96</v>
       </c>
@@ -10435,16 +10546,18 @@
         <v>600000</v>
       </c>
       <c r="AL54">
-        <f>IF(OR(COUNTIF(B54,"*กระบี่*"),COUNTIF(B54,"*จันทบุรี*"),COUNTIF(B54,"*ชุมพร*"),COUNTIF(B54,"*เชียงราย*"),COUNTIF(B54,"*ตรัง*"),COUNTIF(B54,"*นครนายก*"),COUNTIF(B54,"*ปราจีนบุรี*"),COUNTIF(B54,"*พัทลุง*"),COUNTIF(B54,"*ภูเก็ต*"),COUNTIF(B54,"*ยะลา*"),COUNTIF(B54,"*สกลนคร*"),COUNTIF(B54,"*สตูล*"),COUNTIF(B54,"*หนองคาย*"),COUNTIF(B54,"*สุราษฎร์ธานี*"),COUNTIF(B54,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B54,"*ตราด*"),COUNTIF(B54,"*นครพนม*"),COUNTIF(B54,"*นครศรีธรรมราช*"),COUNTIF(B54,"*นราธิวาส*"),COUNTIF(B54,"*บึงกาฬ*"),COUNTIF(B54,"*พังงา*"),COUNTIF(B54,"*ระนอง*"),COUNTIF(B54,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM54">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>25892491.800000001</v>
       </c>
-    </row>
-    <row r="55" spans="1:39">
+      <c r="AN54">
+        <v>6661</v>
+      </c>
+    </row>
+    <row r="55" spans="1:40">
       <c r="A55" t="s">
         <v>94</v>
       </c>
@@ -10567,16 +10680,18 @@
         <v>0</v>
       </c>
       <c r="AL55">
-        <f>IF(OR(COUNTIF(B55,"*กระบี่*"),COUNTIF(B55,"*จันทบุรี*"),COUNTIF(B55,"*ชุมพร*"),COUNTIF(B55,"*เชียงราย*"),COUNTIF(B55,"*ตรัง*"),COUNTIF(B55,"*นครนายก*"),COUNTIF(B55,"*ปราจีนบุรี*"),COUNTIF(B55,"*พัทลุง*"),COUNTIF(B55,"*ภูเก็ต*"),COUNTIF(B55,"*ยะลา*"),COUNTIF(B55,"*สกลนคร*"),COUNTIF(B55,"*สตูล*"),COUNTIF(B55,"*หนองคาย*"),COUNTIF(B55,"*สุราษฎร์ธานี*"),COUNTIF(B55,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B55,"*ตราด*"),COUNTIF(B55,"*นครพนม*"),COUNTIF(B55,"*นครศรีธรรมราช*"),COUNTIF(B55,"*นราธิวาส*"),COUNTIF(B55,"*บึงกาฬ*"),COUNTIF(B55,"*พังงา*"),COUNTIF(B55,"*ระนอง*"),COUNTIF(B55,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM55">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>18861170</v>
       </c>
-    </row>
-    <row r="56" spans="1:39">
+      <c r="AN55">
+        <v>5142.8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:40">
       <c r="A56" t="s">
         <v>96</v>
       </c>
@@ -10699,16 +10814,18 @@
         <v>0</v>
       </c>
       <c r="AL56">
-        <f>IF(OR(COUNTIF(B56,"*กระบี่*"),COUNTIF(B56,"*จันทบุรี*"),COUNTIF(B56,"*ชุมพร*"),COUNTIF(B56,"*เชียงราย*"),COUNTIF(B56,"*ตรัง*"),COUNTIF(B56,"*นครนายก*"),COUNTIF(B56,"*ปราจีนบุรี*"),COUNTIF(B56,"*พัทลุง*"),COUNTIF(B56,"*ภูเก็ต*"),COUNTIF(B56,"*ยะลา*"),COUNTIF(B56,"*สกลนคร*"),COUNTIF(B56,"*สตูล*"),COUNTIF(B56,"*หนองคาย*"),COUNTIF(B56,"*สุราษฎร์ธานี*"),COUNTIF(B56,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B56,"*ตราด*"),COUNTIF(B56,"*นครพนม*"),COUNTIF(B56,"*นครศรีธรรมราช*"),COUNTIF(B56,"*นราธิวาส*"),COUNTIF(B56,"*บึงกาฬ*"),COUNTIF(B56,"*พังงา*"),COUNTIF(B56,"*ระนอง*"),COUNTIF(B56,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM56">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>21938874.260000002</v>
       </c>
-    </row>
-    <row r="57" spans="1:39">
+      <c r="AN56">
+        <v>7791</v>
+      </c>
+    </row>
+    <row r="57" spans="1:40">
       <c r="A57" t="s">
         <v>94</v>
       </c>
@@ -10831,16 +10948,18 @@
         <v>0</v>
       </c>
       <c r="AL57">
-        <f>IF(OR(COUNTIF(B57,"*กระบี่*"),COUNTIF(B57,"*จันทบุรี*"),COUNTIF(B57,"*ชุมพร*"),COUNTIF(B57,"*เชียงราย*"),COUNTIF(B57,"*ตรัง*"),COUNTIF(B57,"*นครนายก*"),COUNTIF(B57,"*ปราจีนบุรี*"),COUNTIF(B57,"*พัทลุง*"),COUNTIF(B57,"*ภูเก็ต*"),COUNTIF(B57,"*ยะลา*"),COUNTIF(B57,"*สกลนคร*"),COUNTIF(B57,"*สตูล*"),COUNTIF(B57,"*หนองคาย*"),COUNTIF(B57,"*สุราษฎร์ธานี*"),COUNTIF(B57,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B57,"*ตราด*"),COUNTIF(B57,"*นครพนม*"),COUNTIF(B57,"*นครศรีธรรมราช*"),COUNTIF(B57,"*นราธิวาส*"),COUNTIF(B57,"*บึงกาฬ*"),COUNTIF(B57,"*พังงา*"),COUNTIF(B57,"*ระนอง*"),COUNTIF(B57,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM57">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>11000590</v>
       </c>
-    </row>
-    <row r="58" spans="1:39">
+      <c r="AN57">
+        <v>9792.1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:40">
       <c r="A58" t="s">
         <v>103</v>
       </c>
@@ -10963,16 +11082,18 @@
         <v>300000</v>
       </c>
       <c r="AL58">
-        <f>IF(OR(COUNTIF(B58,"*กระบี่*"),COUNTIF(B58,"*จันทบุรี*"),COUNTIF(B58,"*ชุมพร*"),COUNTIF(B58,"*เชียงราย*"),COUNTIF(B58,"*ตรัง*"),COUNTIF(B58,"*นครนายก*"),COUNTIF(B58,"*ปราจีนบุรี*"),COUNTIF(B58,"*พัทลุง*"),COUNTIF(B58,"*ภูเก็ต*"),COUNTIF(B58,"*ยะลา*"),COUNTIF(B58,"*สกลนคร*"),COUNTIF(B58,"*สตูล*"),COUNTIF(B58,"*หนองคาย*"),COUNTIF(B58,"*สุราษฎร์ธานี*"),COUNTIF(B58,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B58,"*ตราด*"),COUNTIF(B58,"*นครพนม*"),COUNTIF(B58,"*นครศรีธรรมราช*"),COUNTIF(B58,"*นราธิวาส*"),COUNTIF(B58,"*บึงกาฬ*"),COUNTIF(B58,"*พังงา*"),COUNTIF(B58,"*ระนอง*"),COUNTIF(B58,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM58">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>30530931.02</v>
       </c>
-    </row>
-    <row r="59" spans="1:39">
+      <c r="AN58">
+        <v>5994.5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:40">
       <c r="A59" t="s">
         <v>103</v>
       </c>
@@ -11095,16 +11216,18 @@
         <v>0</v>
       </c>
       <c r="AL59">
-        <f>IF(OR(COUNTIF(B59,"*กระบี่*"),COUNTIF(B59,"*จันทบุรี*"),COUNTIF(B59,"*ชุมพร*"),COUNTIF(B59,"*เชียงราย*"),COUNTIF(B59,"*ตรัง*"),COUNTIF(B59,"*นครนายก*"),COUNTIF(B59,"*ปราจีนบุรี*"),COUNTIF(B59,"*พัทลุง*"),COUNTIF(B59,"*ภูเก็ต*"),COUNTIF(B59,"*ยะลา*"),COUNTIF(B59,"*สกลนคร*"),COUNTIF(B59,"*สตูล*"),COUNTIF(B59,"*หนองคาย*"),COUNTIF(B59,"*สุราษฎร์ธานี*"),COUNTIF(B59,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B59,"*ตราด*"),COUNTIF(B59,"*นครพนม*"),COUNTIF(B59,"*นครศรีธรรมราช*"),COUNTIF(B59,"*นราธิวาส*"),COUNTIF(B59,"*บึงกาฬ*"),COUNTIF(B59,"*พังงา*"),COUNTIF(B59,"*ระนอง*"),COUNTIF(B59,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM59" s="32">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>10792056</v>
       </c>
-    </row>
-    <row r="60" spans="1:39">
+      <c r="AN59">
+        <v>12287.81</v>
+      </c>
+    </row>
+    <row r="60" spans="1:40">
       <c r="A60" t="s">
         <v>103</v>
       </c>
@@ -11227,16 +11350,18 @@
         <v>300000</v>
       </c>
       <c r="AL60">
-        <f>IF(OR(COUNTIF(B60,"*กระบี่*"),COUNTIF(B60,"*จันทบุรี*"),COUNTIF(B60,"*ชุมพร*"),COUNTIF(B60,"*เชียงราย*"),COUNTIF(B60,"*ตรัง*"),COUNTIF(B60,"*นครนายก*"),COUNTIF(B60,"*ปราจีนบุรี*"),COUNTIF(B60,"*พัทลุง*"),COUNTIF(B60,"*ภูเก็ต*"),COUNTIF(B60,"*ยะลา*"),COUNTIF(B60,"*สกลนคร*"),COUNTIF(B60,"*สตูล*"),COUNTIF(B60,"*หนองคาย*"),COUNTIF(B60,"*สุราษฎร์ธานี*"),COUNTIF(B60,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B60,"*ตราด*"),COUNTIF(B60,"*นครพนม*"),COUNTIF(B60,"*นครศรีธรรมราช*"),COUNTIF(B60,"*นราธิวาส*"),COUNTIF(B60,"*บึงกาฬ*"),COUNTIF(B60,"*พังงา*"),COUNTIF(B60,"*ระนอง*"),COUNTIF(B60,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM60">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>9142855</v>
       </c>
-    </row>
-    <row r="61" spans="1:39">
+      <c r="AN60">
+        <v>9503</v>
+      </c>
+    </row>
+    <row r="61" spans="1:40">
       <c r="A61" t="s">
         <v>103</v>
       </c>
@@ -11359,16 +11484,18 @@
         <v>300000</v>
       </c>
       <c r="AL61">
-        <f>IF(OR(COUNTIF(B61,"*กระบี่*"),COUNTIF(B61,"*จันทบุรี*"),COUNTIF(B61,"*ชุมพร*"),COUNTIF(B61,"*เชียงราย*"),COUNTIF(B61,"*ตรัง*"),COUNTIF(B61,"*นครนายก*"),COUNTIF(B61,"*ปราจีนบุรี*"),COUNTIF(B61,"*พัทลุง*"),COUNTIF(B61,"*ภูเก็ต*"),COUNTIF(B61,"*ยะลา*"),COUNTIF(B61,"*สกลนคร*"),COUNTIF(B61,"*สตูล*"),COUNTIF(B61,"*หนองคาย*"),COUNTIF(B61,"*สุราษฎร์ธานี*"),COUNTIF(B61,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B61,"*ตราด*"),COUNTIF(B61,"*นครพนม*"),COUNTIF(B61,"*นครศรีธรรมราช*"),COUNTIF(B61,"*นราธิวาส*"),COUNTIF(B61,"*บึงกาฬ*"),COUNTIF(B61,"*พังงา*"),COUNTIF(B61,"*ระนอง*"),COUNTIF(B61,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM61">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>8114437.2000000002</v>
       </c>
-    </row>
-    <row r="62" spans="1:39">
+      <c r="AN61">
+        <v>4362</v>
+      </c>
+    </row>
+    <row r="62" spans="1:40">
       <c r="A62" t="s">
         <v>103</v>
       </c>
@@ -11491,16 +11618,18 @@
         <v>300000</v>
       </c>
       <c r="AL62">
-        <f>IF(OR(COUNTIF(B62,"*กระบี่*"),COUNTIF(B62,"*จันทบุรี*"),COUNTIF(B62,"*ชุมพร*"),COUNTIF(B62,"*เชียงราย*"),COUNTIF(B62,"*ตรัง*"),COUNTIF(B62,"*นครนายก*"),COUNTIF(B62,"*ปราจีนบุรี*"),COUNTIF(B62,"*พัทลุง*"),COUNTIF(B62,"*ภูเก็ต*"),COUNTIF(B62,"*ยะลา*"),COUNTIF(B62,"*สกลนคร*"),COUNTIF(B62,"*สตูล*"),COUNTIF(B62,"*หนองคาย*"),COUNTIF(B62,"*สุราษฎร์ธานี*"),COUNTIF(B62,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B62,"*ตราด*"),COUNTIF(B62,"*นครพนม*"),COUNTIF(B62,"*นครศรีธรรมราช*"),COUNTIF(B62,"*นราธิวาส*"),COUNTIF(B62,"*บึงกาฬ*"),COUNTIF(B62,"*พังงา*"),COUNTIF(B62,"*ระนอง*"),COUNTIF(B62,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM62">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>4802893</v>
       </c>
-    </row>
-    <row r="63" spans="1:39">
+      <c r="AN62">
+        <v>5731.3</v>
+      </c>
+    </row>
+    <row r="63" spans="1:40">
       <c r="A63" t="s">
         <v>103</v>
       </c>
@@ -11623,16 +11752,18 @@
         <v>0</v>
       </c>
       <c r="AL63">
-        <f>IF(OR(COUNTIF(B63,"*กระบี่*"),COUNTIF(B63,"*จันทบุรี*"),COUNTIF(B63,"*ชุมพร*"),COUNTIF(B63,"*เชียงราย*"),COUNTIF(B63,"*ตรัง*"),COUNTIF(B63,"*นครนายก*"),COUNTIF(B63,"*ปราจีนบุรี*"),COUNTIF(B63,"*พัทลุง*"),COUNTIF(B63,"*ภูเก็ต*"),COUNTIF(B63,"*ยะลา*"),COUNTIF(B63,"*สกลนคร*"),COUNTIF(B63,"*สตูล*"),COUNTIF(B63,"*หนองคาย*"),COUNTIF(B63,"*สุราษฎร์ธานี*"),COUNTIF(B63,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B63,"*ตราด*"),COUNTIF(B63,"*นครพนม*"),COUNTIF(B63,"*นครศรีธรรมราช*"),COUNTIF(B63,"*นราธิวาส*"),COUNTIF(B63,"*บึงกาฬ*"),COUNTIF(B63,"*พังงา*"),COUNTIF(B63,"*ระนอง*"),COUNTIF(B63,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM63" s="32">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>16237561.5</v>
       </c>
-    </row>
-    <row r="64" spans="1:39">
+      <c r="AN63">
+        <v>5050</v>
+      </c>
+    </row>
+    <row r="64" spans="1:40">
       <c r="A64" t="s">
         <v>103</v>
       </c>
@@ -11755,16 +11886,18 @@
         <v>600000</v>
       </c>
       <c r="AL64">
-        <f>IF(OR(COUNTIF(B64,"*กระบี่*"),COUNTIF(B64,"*จันทบุรี*"),COUNTIF(B64,"*ชุมพร*"),COUNTIF(B64,"*เชียงราย*"),COUNTIF(B64,"*ตรัง*"),COUNTIF(B64,"*นครนายก*"),COUNTIF(B64,"*ปราจีนบุรี*"),COUNTIF(B64,"*พัทลุง*"),COUNTIF(B64,"*ภูเก็ต*"),COUNTIF(B64,"*ยะลา*"),COUNTIF(B64,"*สกลนคร*"),COUNTIF(B64,"*สตูล*"),COUNTIF(B64,"*หนองคาย*"),COUNTIF(B64,"*สุราษฎร์ธานี*"),COUNTIF(B64,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B64,"*ตราด*"),COUNTIF(B64,"*นครพนม*"),COUNTIF(B64,"*นครศรีธรรมราช*"),COUNTIF(B64,"*นราธิวาส*"),COUNTIF(B64,"*บึงกาฬ*"),COUNTIF(B64,"*พังงา*"),COUNTIF(B64,"*ระนอง*"),COUNTIF(B64,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM64">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>10140437</v>
       </c>
-    </row>
-    <row r="65" spans="1:39">
+      <c r="AN64">
+        <v>5643.9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:40">
       <c r="A65" t="s">
         <v>111</v>
       </c>
@@ -11887,16 +12020,18 @@
         <v>0</v>
       </c>
       <c r="AL65">
-        <f>IF(OR(COUNTIF(B65,"*กระบี่*"),COUNTIF(B65,"*จันทบุรี*"),COUNTIF(B65,"*ชุมพร*"),COUNTIF(B65,"*เชียงราย*"),COUNTIF(B65,"*ตรัง*"),COUNTIF(B65,"*นครนายก*"),COUNTIF(B65,"*ปราจีนบุรี*"),COUNTIF(B65,"*พัทลุง*"),COUNTIF(B65,"*ภูเก็ต*"),COUNTIF(B65,"*ยะลา*"),COUNTIF(B65,"*สกลนคร*"),COUNTIF(B65,"*สตูล*"),COUNTIF(B65,"*หนองคาย*"),COUNTIF(B65,"*สุราษฎร์ธานี*"),COUNTIF(B65,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B65,"*ตราด*"),COUNTIF(B65,"*นครพนม*"),COUNTIF(B65,"*นครศรีธรรมราช*"),COUNTIF(B65,"*นราธิวาส*"),COUNTIF(B65,"*บึงกาฬ*"),COUNTIF(B65,"*พังงา*"),COUNTIF(B65,"*ระนอง*"),COUNTIF(B65,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM65">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>29465698.710000001</v>
       </c>
-    </row>
-    <row r="66" spans="1:39">
+      <c r="AN65">
+        <v>8265</v>
+      </c>
+    </row>
+    <row r="66" spans="1:40">
       <c r="A66" t="s">
         <v>111</v>
       </c>
@@ -12019,7 +12154,7 @@
         <v>300000</v>
       </c>
       <c r="AL66">
-        <f>IF(OR(COUNTIF(B66,"*กระบี่*"),COUNTIF(B66,"*จันทบุรี*"),COUNTIF(B66,"*ชุมพร*"),COUNTIF(B66,"*เชียงราย*"),COUNTIF(B66,"*ตรัง*"),COUNTIF(B66,"*นครนายก*"),COUNTIF(B66,"*ปราจีนบุรี*"),COUNTIF(B66,"*พัทลุง*"),COUNTIF(B66,"*ภูเก็ต*"),COUNTIF(B66,"*ยะลา*"),COUNTIF(B66,"*สกลนคร*"),COUNTIF(B66,"*สตูล*"),COUNTIF(B66,"*หนองคาย*"),COUNTIF(B66,"*สุราษฎร์ธานี*"),COUNTIF(B66,"*ปัตตานี*")),2,
+        <f t="shared" ref="AL66:AL97" si="2">IF(OR(COUNTIF(B66,"*กระบี่*"),COUNTIF(B66,"*จันทบุรี*"),COUNTIF(B66,"*ชุมพร*"),COUNTIF(B66,"*เชียงราย*"),COUNTIF(B66,"*ตรัง*"),COUNTIF(B66,"*นครนายก*"),COUNTIF(B66,"*ปราจีนบุรี*"),COUNTIF(B66,"*พัทลุง*"),COUNTIF(B66,"*ภูเก็ต*"),COUNTIF(B66,"*ยะลา*"),COUNTIF(B66,"*สกลนคร*"),COUNTIF(B66,"*สตูล*"),COUNTIF(B66,"*หนองคาย*"),COUNTIF(B66,"*สุราษฎร์ธานี*"),COUNTIF(B66,"*ปัตตานี*")),2,
 IF(OR(COUNTIF(B66,"*ตราด*"),COUNTIF(B66,"*นครพนม*"),COUNTIF(B66,"*นครศรีธรรมราช*"),COUNTIF(B66,"*นราธิวาส*"),COUNTIF(B66,"*บึงกาฬ*"),COUNTIF(B66,"*พังงา*"),COUNTIF(B66,"*ระนอง*"),COUNTIF(B66,"*สงขลา*")),4,0))</f>
         <v>2</v>
       </c>
@@ -12027,8 +12162,11 @@
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>15692770.6</v>
       </c>
-    </row>
-    <row r="67" spans="1:39">
+      <c r="AN66">
+        <v>7504.5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:40">
       <c r="A67" t="s">
         <v>111</v>
       </c>
@@ -12151,16 +12289,18 @@
         <v>0</v>
       </c>
       <c r="AL67">
-        <f>IF(OR(COUNTIF(B67,"*กระบี่*"),COUNTIF(B67,"*จันทบุรี*"),COUNTIF(B67,"*ชุมพร*"),COUNTIF(B67,"*เชียงราย*"),COUNTIF(B67,"*ตรัง*"),COUNTIF(B67,"*นครนายก*"),COUNTIF(B67,"*ปราจีนบุรี*"),COUNTIF(B67,"*พัทลุง*"),COUNTIF(B67,"*ภูเก็ต*"),COUNTIF(B67,"*ยะลา*"),COUNTIF(B67,"*สกลนคร*"),COUNTIF(B67,"*สตูล*"),COUNTIF(B67,"*หนองคาย*"),COUNTIF(B67,"*สุราษฎร์ธานี*"),COUNTIF(B67,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B67,"*ตราด*"),COUNTIF(B67,"*นครพนม*"),COUNTIF(B67,"*นครศรีธรรมราช*"),COUNTIF(B67,"*นราธิวาส*"),COUNTIF(B67,"*บึงกาฬ*"),COUNTIF(B67,"*พังงา*"),COUNTIF(B67,"*ระนอง*"),COUNTIF(B67,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM67">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>15740359.6</v>
       </c>
-    </row>
-    <row r="68" spans="1:39">
+      <c r="AN67">
+        <v>6179</v>
+      </c>
+    </row>
+    <row r="68" spans="1:40">
       <c r="A68" t="s">
         <v>111</v>
       </c>
@@ -12283,16 +12423,18 @@
         <v>1200000</v>
       </c>
       <c r="AL68">
-        <f>IF(OR(COUNTIF(B68,"*กระบี่*"),COUNTIF(B68,"*จันทบุรี*"),COUNTIF(B68,"*ชุมพร*"),COUNTIF(B68,"*เชียงราย*"),COUNTIF(B68,"*ตรัง*"),COUNTIF(B68,"*นครนายก*"),COUNTIF(B68,"*ปราจีนบุรี*"),COUNTIF(B68,"*พัทลุง*"),COUNTIF(B68,"*ภูเก็ต*"),COUNTIF(B68,"*ยะลา*"),COUNTIF(B68,"*สกลนคร*"),COUNTIF(B68,"*สตูล*"),COUNTIF(B68,"*หนองคาย*"),COUNTIF(B68,"*สุราษฎร์ธานี*"),COUNTIF(B68,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B68,"*ตราด*"),COUNTIF(B68,"*นครพนม*"),COUNTIF(B68,"*นครศรีธรรมราช*"),COUNTIF(B68,"*นราธิวาส*"),COUNTIF(B68,"*บึงกาฬ*"),COUNTIF(B68,"*พังงา*"),COUNTIF(B68,"*ระนอง*"),COUNTIF(B68,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM68">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>20341909.600000001</v>
       </c>
-    </row>
-    <row r="69" spans="1:39">
+      <c r="AN68">
+        <v>6168.8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:40">
       <c r="A69" t="s">
         <v>111</v>
       </c>
@@ -12415,16 +12557,18 @@
         <v>0</v>
       </c>
       <c r="AL69">
-        <f>IF(OR(COUNTIF(B69,"*กระบี่*"),COUNTIF(B69,"*จันทบุรี*"),COUNTIF(B69,"*ชุมพร*"),COUNTIF(B69,"*เชียงราย*"),COUNTIF(B69,"*ตรัง*"),COUNTIF(B69,"*นครนายก*"),COUNTIF(B69,"*ปราจีนบุรี*"),COUNTIF(B69,"*พัทลุง*"),COUNTIF(B69,"*ภูเก็ต*"),COUNTIF(B69,"*ยะลา*"),COUNTIF(B69,"*สกลนคร*"),COUNTIF(B69,"*สตูล*"),COUNTIF(B69,"*หนองคาย*"),COUNTIF(B69,"*สุราษฎร์ธานี*"),COUNTIF(B69,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B69,"*ตราด*"),COUNTIF(B69,"*นครพนม*"),COUNTIF(B69,"*นครศรีธรรมราช*"),COUNTIF(B69,"*นราธิวาส*"),COUNTIF(B69,"*บึงกาฬ*"),COUNTIF(B69,"*พังงา*"),COUNTIF(B69,"*ระนอง*"),COUNTIF(B69,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="AM69" s="32">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>22723883</v>
       </c>
-    </row>
-    <row r="70" spans="1:39">
+      <c r="AN69">
+        <v>7616</v>
+      </c>
+    </row>
+    <row r="70" spans="1:40">
       <c r="A70" t="s">
         <v>111</v>
       </c>
@@ -12547,16 +12691,18 @@
         <v>0</v>
       </c>
       <c r="AL70">
-        <f>IF(OR(COUNTIF(B70,"*กระบี่*"),COUNTIF(B70,"*จันทบุรี*"),COUNTIF(B70,"*ชุมพร*"),COUNTIF(B70,"*เชียงราย*"),COUNTIF(B70,"*ตรัง*"),COUNTIF(B70,"*นครนายก*"),COUNTIF(B70,"*ปราจีนบุรี*"),COUNTIF(B70,"*พัทลุง*"),COUNTIF(B70,"*ภูเก็ต*"),COUNTIF(B70,"*ยะลา*"),COUNTIF(B70,"*สกลนคร*"),COUNTIF(B70,"*สตูล*"),COUNTIF(B70,"*หนองคาย*"),COUNTIF(B70,"*สุราษฎร์ธานี*"),COUNTIF(B70,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B70,"*ตราด*"),COUNTIF(B70,"*นครพนม*"),COUNTIF(B70,"*นครศรีธรรมราช*"),COUNTIF(B70,"*นราธิวาส*"),COUNTIF(B70,"*บึงกาฬ*"),COUNTIF(B70,"*พังงา*"),COUNTIF(B70,"*ระนอง*"),COUNTIF(B70,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM70">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>15582254</v>
       </c>
-    </row>
-    <row r="71" spans="1:39">
+      <c r="AN70">
+        <v>5569</v>
+      </c>
+    </row>
+    <row r="71" spans="1:40">
       <c r="A71" t="s">
         <v>118</v>
       </c>
@@ -12679,16 +12825,18 @@
         <v>0</v>
       </c>
       <c r="AL71">
-        <f>IF(OR(COUNTIF(B71,"*กระบี่*"),COUNTIF(B71,"*จันทบุรี*"),COUNTIF(B71,"*ชุมพร*"),COUNTIF(B71,"*เชียงราย*"),COUNTIF(B71,"*ตรัง*"),COUNTIF(B71,"*นครนายก*"),COUNTIF(B71,"*ปราจีนบุรี*"),COUNTIF(B71,"*พัทลุง*"),COUNTIF(B71,"*ภูเก็ต*"),COUNTIF(B71,"*ยะลา*"),COUNTIF(B71,"*สกลนคร*"),COUNTIF(B71,"*สตูล*"),COUNTIF(B71,"*หนองคาย*"),COUNTIF(B71,"*สุราษฎร์ธานี*"),COUNTIF(B71,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B71,"*ตราด*"),COUNTIF(B71,"*นครพนม*"),COUNTIF(B71,"*นครศรีธรรมราช*"),COUNTIF(B71,"*นราธิวาส*"),COUNTIF(B71,"*บึงกาฬ*"),COUNTIF(B71,"*พังงา*"),COUNTIF(B71,"*ระนอง*"),COUNTIF(B71,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM71" s="32">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>11537730</v>
       </c>
-    </row>
-    <row r="72" spans="1:39">
+      <c r="AN71">
+        <v>6359.23</v>
+      </c>
+    </row>
+    <row r="72" spans="1:40">
       <c r="A72" t="s">
         <v>118</v>
       </c>
@@ -12811,16 +12959,18 @@
         <v>0</v>
       </c>
       <c r="AL72">
-        <f>IF(OR(COUNTIF(B72,"*กระบี่*"),COUNTIF(B72,"*จันทบุรี*"),COUNTIF(B72,"*ชุมพร*"),COUNTIF(B72,"*เชียงราย*"),COUNTIF(B72,"*ตรัง*"),COUNTIF(B72,"*นครนายก*"),COUNTIF(B72,"*ปราจีนบุรี*"),COUNTIF(B72,"*พัทลุง*"),COUNTIF(B72,"*ภูเก็ต*"),COUNTIF(B72,"*ยะลา*"),COUNTIF(B72,"*สกลนคร*"),COUNTIF(B72,"*สตูล*"),COUNTIF(B72,"*หนองคาย*"),COUNTIF(B72,"*สุราษฎร์ธานี*"),COUNTIF(B72,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B72,"*ตราด*"),COUNTIF(B72,"*นครพนม*"),COUNTIF(B72,"*นครศรีธรรมราช*"),COUNTIF(B72,"*นราธิวาส*"),COUNTIF(B72,"*บึงกาฬ*"),COUNTIF(B72,"*พังงา*"),COUNTIF(B72,"*ระนอง*"),COUNTIF(B72,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM72">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>19196889</v>
       </c>
-    </row>
-    <row r="73" spans="1:39">
+      <c r="AN72">
+        <v>7181</v>
+      </c>
+    </row>
+    <row r="73" spans="1:40">
       <c r="A73" t="s">
         <v>118</v>
       </c>
@@ -12943,16 +13093,18 @@
         <v>300000</v>
       </c>
       <c r="AL73">
-        <f>IF(OR(COUNTIF(B73,"*กระบี่*"),COUNTIF(B73,"*จันทบุรี*"),COUNTIF(B73,"*ชุมพร*"),COUNTIF(B73,"*เชียงราย*"),COUNTIF(B73,"*ตรัง*"),COUNTIF(B73,"*นครนายก*"),COUNTIF(B73,"*ปราจีนบุรี*"),COUNTIF(B73,"*พัทลุง*"),COUNTIF(B73,"*ภูเก็ต*"),COUNTIF(B73,"*ยะลา*"),COUNTIF(B73,"*สกลนคร*"),COUNTIF(B73,"*สตูล*"),COUNTIF(B73,"*หนองคาย*"),COUNTIF(B73,"*สุราษฎร์ธานี*"),COUNTIF(B73,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B73,"*ตราด*"),COUNTIF(B73,"*นครพนม*"),COUNTIF(B73,"*นครศรีธรรมราช*"),COUNTIF(B73,"*นราธิวาส*"),COUNTIF(B73,"*บึงกาฬ*"),COUNTIF(B73,"*พังงา*"),COUNTIF(B73,"*ระนอง*"),COUNTIF(B73,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM73">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>27207523.800000001</v>
       </c>
-    </row>
-    <row r="74" spans="1:39">
+      <c r="AN73">
+        <v>4814.6000000000004</v>
+      </c>
+    </row>
+    <row r="74" spans="1:40">
       <c r="A74" t="s">
         <v>118</v>
       </c>
@@ -13060,16 +13212,18 @@
         <v>0</v>
       </c>
       <c r="AL74">
-        <f>IF(OR(COUNTIF(B74,"*กระบี่*"),COUNTIF(B74,"*จันทบุรี*"),COUNTIF(B74,"*ชุมพร*"),COUNTIF(B74,"*เชียงราย*"),COUNTIF(B74,"*ตรัง*"),COUNTIF(B74,"*นครนายก*"),COUNTIF(B74,"*ปราจีนบุรี*"),COUNTIF(B74,"*พัทลุง*"),COUNTIF(B74,"*ภูเก็ต*"),COUNTIF(B74,"*ยะลา*"),COUNTIF(B74,"*สกลนคร*"),COUNTIF(B74,"*สตูล*"),COUNTIF(B74,"*หนองคาย*"),COUNTIF(B74,"*สุราษฎร์ธานี*"),COUNTIF(B74,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B74,"*ตราด*"),COUNTIF(B74,"*นครพนม*"),COUNTIF(B74,"*นครศรีธรรมราช*"),COUNTIF(B74,"*นราธิวาส*"),COUNTIF(B74,"*บึงกาฬ*"),COUNTIF(B74,"*พังงา*"),COUNTIF(B74,"*ระนอง*"),COUNTIF(B74,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM74">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>8083728</v>
       </c>
-    </row>
-    <row r="75" spans="1:39">
+      <c r="AN74">
+        <v>3574.7</v>
+      </c>
+    </row>
+    <row r="75" spans="1:40">
       <c r="A75" t="s">
         <v>94</v>
       </c>
@@ -13192,20 +13346,22 @@
         <v>0</v>
       </c>
       <c r="AL75">
-        <f>IF(OR(COUNTIF(B75,"*กระบี่*"),COUNTIF(B75,"*จันทบุรี*"),COUNTIF(B75,"*ชุมพร*"),COUNTIF(B75,"*เชียงราย*"),COUNTIF(B75,"*ตรัง*"),COUNTIF(B75,"*นครนายก*"),COUNTIF(B75,"*ปราจีนบุรี*"),COUNTIF(B75,"*พัทลุง*"),COUNTIF(B75,"*ภูเก็ต*"),COUNTIF(B75,"*ยะลา*"),COUNTIF(B75,"*สกลนคร*"),COUNTIF(B75,"*สตูล*"),COUNTIF(B75,"*หนองคาย*"),COUNTIF(B75,"*สุราษฎร์ธานี*"),COUNTIF(B75,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B75,"*ตราด*"),COUNTIF(B75,"*นครพนม*"),COUNTIF(B75,"*นครศรีธรรมราช*"),COUNTIF(B75,"*นราธิวาส*"),COUNTIF(B75,"*บึงกาฬ*"),COUNTIF(B75,"*พังงา*"),COUNTIF(B75,"*ระนอง*"),COUNTIF(B75,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM75">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>10721782.49</v>
       </c>
-    </row>
-    <row r="76" spans="1:39">
+      <c r="AN75">
+        <v>7473.51</v>
+      </c>
+    </row>
+    <row r="76" spans="1:40">
       <c r="A76" t="s">
         <v>94</v>
       </c>
-      <c r="B76" s="82" t="s">
+      <c r="B76" t="s">
         <v>124</v>
       </c>
       <c r="C76" s="39">
@@ -13309,16 +13465,18 @@
         <v>300000</v>
       </c>
       <c r="AL76">
-        <f>IF(OR(COUNTIF(B76,"*กระบี่*"),COUNTIF(B76,"*จันทบุรี*"),COUNTIF(B76,"*ชุมพร*"),COUNTIF(B76,"*เชียงราย*"),COUNTIF(B76,"*ตรัง*"),COUNTIF(B76,"*นครนายก*"),COUNTIF(B76,"*ปราจีนบุรี*"),COUNTIF(B76,"*พัทลุง*"),COUNTIF(B76,"*ภูเก็ต*"),COUNTIF(B76,"*ยะลา*"),COUNTIF(B76,"*สกลนคร*"),COUNTIF(B76,"*สตูล*"),COUNTIF(B76,"*หนองคาย*"),COUNTIF(B76,"*สุราษฎร์ธานี*"),COUNTIF(B76,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B76,"*ตราด*"),COUNTIF(B76,"*นครพนม*"),COUNTIF(B76,"*นครศรีธรรมราช*"),COUNTIF(B76,"*นราธิวาส*"),COUNTIF(B76,"*บึงกาฬ*"),COUNTIF(B76,"*พังงา*"),COUNTIF(B76,"*ระนอง*"),COUNTIF(B76,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM76">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>13851183.5</v>
       </c>
-    </row>
-    <row r="77" spans="1:39">
+      <c r="AN76">
+        <v>5151</v>
+      </c>
+    </row>
+    <row r="77" spans="1:40">
       <c r="A77" t="s">
         <v>125</v>
       </c>
@@ -13441,16 +13599,18 @@
         <v>600000</v>
       </c>
       <c r="AL77">
-        <f>IF(OR(COUNTIF(B77,"*กระบี่*"),COUNTIF(B77,"*จันทบุรี*"),COUNTIF(B77,"*ชุมพร*"),COUNTIF(B77,"*เชียงราย*"),COUNTIF(B77,"*ตรัง*"),COUNTIF(B77,"*นครนายก*"),COUNTIF(B77,"*ปราจีนบุรี*"),COUNTIF(B77,"*พัทลุง*"),COUNTIF(B77,"*ภูเก็ต*"),COUNTIF(B77,"*ยะลา*"),COUNTIF(B77,"*สกลนคร*"),COUNTIF(B77,"*สตูล*"),COUNTIF(B77,"*หนองคาย*"),COUNTIF(B77,"*สุราษฎร์ธานี*"),COUNTIF(B77,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B77,"*ตราด*"),COUNTIF(B77,"*นครพนม*"),COUNTIF(B77,"*นครศรีธรรมราช*"),COUNTIF(B77,"*นราธิวาส*"),COUNTIF(B77,"*บึงกาฬ*"),COUNTIF(B77,"*พังงา*"),COUNTIF(B77,"*ระนอง*"),COUNTIF(B77,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM77">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>13414190</v>
       </c>
-    </row>
-    <row r="78" spans="1:39">
+      <c r="AN77">
+        <v>6868.54</v>
+      </c>
+    </row>
+    <row r="78" spans="1:40">
       <c r="A78" t="s">
         <v>125</v>
       </c>
@@ -13573,16 +13733,18 @@
         <v>0</v>
       </c>
       <c r="AL78">
-        <f>IF(OR(COUNTIF(B78,"*กระบี่*"),COUNTIF(B78,"*จันทบุรี*"),COUNTIF(B78,"*ชุมพร*"),COUNTIF(B78,"*เชียงราย*"),COUNTIF(B78,"*ตรัง*"),COUNTIF(B78,"*นครนายก*"),COUNTIF(B78,"*ปราจีนบุรี*"),COUNTIF(B78,"*พัทลุง*"),COUNTIF(B78,"*ภูเก็ต*"),COUNTIF(B78,"*ยะลา*"),COUNTIF(B78,"*สกลนคร*"),COUNTIF(B78,"*สตูล*"),COUNTIF(B78,"*หนองคาย*"),COUNTIF(B78,"*สุราษฎร์ธานี*"),COUNTIF(B78,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B78,"*ตราด*"),COUNTIF(B78,"*นครพนม*"),COUNTIF(B78,"*นครศรีธรรมราช*"),COUNTIF(B78,"*นราธิวาส*"),COUNTIF(B78,"*บึงกาฬ*"),COUNTIF(B78,"*พังงา*"),COUNTIF(B78,"*ระนอง*"),COUNTIF(B78,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM78">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>4604279.46</v>
       </c>
-    </row>
-    <row r="79" spans="1:39">
+      <c r="AN78">
+        <v>12392.234</v>
+      </c>
+    </row>
+    <row r="79" spans="1:40">
       <c r="A79" t="s">
         <v>125</v>
       </c>
@@ -13705,16 +13867,18 @@
         <v>900000</v>
       </c>
       <c r="AL79">
-        <f>IF(OR(COUNTIF(B79,"*กระบี่*"),COUNTIF(B79,"*จันทบุรี*"),COUNTIF(B79,"*ชุมพร*"),COUNTIF(B79,"*เชียงราย*"),COUNTIF(B79,"*ตรัง*"),COUNTIF(B79,"*นครนายก*"),COUNTIF(B79,"*ปราจีนบุรี*"),COUNTIF(B79,"*พัทลุง*"),COUNTIF(B79,"*ภูเก็ต*"),COUNTIF(B79,"*ยะลา*"),COUNTIF(B79,"*สกลนคร*"),COUNTIF(B79,"*สตูล*"),COUNTIF(B79,"*หนองคาย*"),COUNTIF(B79,"*สุราษฎร์ธานี*"),COUNTIF(B79,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B79,"*ตราด*"),COUNTIF(B79,"*นครพนม*"),COUNTIF(B79,"*นครศรีธรรมราช*"),COUNTIF(B79,"*นราธิวาส*"),COUNTIF(B79,"*บึงกาฬ*"),COUNTIF(B79,"*พังงา*"),COUNTIF(B79,"*ระนอง*"),COUNTIF(B79,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM79">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>8886123.0600000005</v>
       </c>
-    </row>
-    <row r="80" spans="1:39">
+      <c r="AN79">
+        <v>5434</v>
+      </c>
+    </row>
+    <row r="80" spans="1:40">
       <c r="A80" t="s">
         <v>129</v>
       </c>
@@ -13837,16 +14001,18 @@
         <v>0</v>
       </c>
       <c r="AL80">
-        <f>IF(OR(COUNTIF(B80,"*กระบี่*"),COUNTIF(B80,"*จันทบุรี*"),COUNTIF(B80,"*ชุมพร*"),COUNTIF(B80,"*เชียงราย*"),COUNTIF(B80,"*ตรัง*"),COUNTIF(B80,"*นครนายก*"),COUNTIF(B80,"*ปราจีนบุรี*"),COUNTIF(B80,"*พัทลุง*"),COUNTIF(B80,"*ภูเก็ต*"),COUNTIF(B80,"*ยะลา*"),COUNTIF(B80,"*สกลนคร*"),COUNTIF(B80,"*สตูล*"),COUNTIF(B80,"*หนองคาย*"),COUNTIF(B80,"*สุราษฎร์ธานี*"),COUNTIF(B80,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B80,"*ตราด*"),COUNTIF(B80,"*นครพนม*"),COUNTIF(B80,"*นครศรีธรรมราช*"),COUNTIF(B80,"*นราธิวาส*"),COUNTIF(B80,"*บึงกาฬ*"),COUNTIF(B80,"*พังงา*"),COUNTIF(B80,"*ระนอง*"),COUNTIF(B80,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM80">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>16635212</v>
       </c>
-    </row>
-    <row r="81" spans="1:39">
+      <c r="AN80">
+        <v>7425.37</v>
+      </c>
+    </row>
+    <row r="81" spans="1:40">
       <c r="A81" t="s">
         <v>125</v>
       </c>
@@ -13969,16 +14135,18 @@
         <v>0</v>
       </c>
       <c r="AL81">
-        <f>IF(OR(COUNTIF(B81,"*กระบี่*"),COUNTIF(B81,"*จันทบุรี*"),COUNTIF(B81,"*ชุมพร*"),COUNTIF(B81,"*เชียงราย*"),COUNTIF(B81,"*ตรัง*"),COUNTIF(B81,"*นครนายก*"),COUNTIF(B81,"*ปราจีนบุรี*"),COUNTIF(B81,"*พัทลุง*"),COUNTIF(B81,"*ภูเก็ต*"),COUNTIF(B81,"*ยะลา*"),COUNTIF(B81,"*สกลนคร*"),COUNTIF(B81,"*สตูล*"),COUNTIF(B81,"*หนองคาย*"),COUNTIF(B81,"*สุราษฎร์ธานี*"),COUNTIF(B81,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B81,"*ตราด*"),COUNTIF(B81,"*นครพนม*"),COUNTIF(B81,"*นครศรีธรรมราช*"),COUNTIF(B81,"*นราธิวาส*"),COUNTIF(B81,"*บึงกาฬ*"),COUNTIF(B81,"*พังงา*"),COUNTIF(B81,"*ระนอง*"),COUNTIF(B81,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM81">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>5433140</v>
       </c>
-    </row>
-    <row r="82" spans="1:39">
+      <c r="AN81">
+        <v>5519.5</v>
+      </c>
+    </row>
+    <row r="82" spans="1:40">
       <c r="A82" t="s">
         <v>125</v>
       </c>
@@ -14101,16 +14269,18 @@
         <v>1200000</v>
       </c>
       <c r="AL82">
-        <f>IF(OR(COUNTIF(B82,"*กระบี่*"),COUNTIF(B82,"*จันทบุรี*"),COUNTIF(B82,"*ชุมพร*"),COUNTIF(B82,"*เชียงราย*"),COUNTIF(B82,"*ตรัง*"),COUNTIF(B82,"*นครนายก*"),COUNTIF(B82,"*ปราจีนบุรี*"),COUNTIF(B82,"*พัทลุง*"),COUNTIF(B82,"*ภูเก็ต*"),COUNTIF(B82,"*ยะลา*"),COUNTIF(B82,"*สกลนคร*"),COUNTIF(B82,"*สตูล*"),COUNTIF(B82,"*หนองคาย*"),COUNTIF(B82,"*สุราษฎร์ธานี*"),COUNTIF(B82,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B82,"*ตราด*"),COUNTIF(B82,"*นครพนม*"),COUNTIF(B82,"*นครศรีธรรมราช*"),COUNTIF(B82,"*นราธิวาส*"),COUNTIF(B82,"*บึงกาฬ*"),COUNTIF(B82,"*พังงา*"),COUNTIF(B82,"*ระนอง*"),COUNTIF(B82,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="AM82">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>15085067.1</v>
       </c>
-    </row>
-    <row r="83" spans="1:39">
+      <c r="AN82">
+        <v>8958.1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:40">
       <c r="A83" t="s">
         <v>125</v>
       </c>
@@ -14227,16 +14397,18 @@
         <v>300000</v>
       </c>
       <c r="AL83">
-        <f>IF(OR(COUNTIF(B83,"*กระบี่*"),COUNTIF(B83,"*จันทบุรี*"),COUNTIF(B83,"*ชุมพร*"),COUNTIF(B83,"*เชียงราย*"),COUNTIF(B83,"*ตรัง*"),COUNTIF(B83,"*นครนายก*"),COUNTIF(B83,"*ปราจีนบุรี*"),COUNTIF(B83,"*พัทลุง*"),COUNTIF(B83,"*ภูเก็ต*"),COUNTIF(B83,"*ยะลา*"),COUNTIF(B83,"*สกลนคร*"),COUNTIF(B83,"*สตูล*"),COUNTIF(B83,"*หนองคาย*"),COUNTIF(B83,"*สุราษฎร์ธานี*"),COUNTIF(B83,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B83,"*ตราด*"),COUNTIF(B83,"*นครพนม*"),COUNTIF(B83,"*นครศรีธรรมราช*"),COUNTIF(B83,"*นราธิวาส*"),COUNTIF(B83,"*บึงกาฬ*"),COUNTIF(B83,"*พังงา*"),COUNTIF(B83,"*ระนอง*"),COUNTIF(B83,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM83">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>12149336</v>
       </c>
-    </row>
-    <row r="84" spans="1:39">
+      <c r="AN83">
+        <v>3963</v>
+      </c>
+    </row>
+    <row r="84" spans="1:40">
       <c r="A84" t="s">
         <v>134</v>
       </c>
@@ -14359,16 +14531,18 @@
         <v>0</v>
       </c>
       <c r="AL84">
-        <f>IF(OR(COUNTIF(B84,"*กระบี่*"),COUNTIF(B84,"*จันทบุรี*"),COUNTIF(B84,"*ชุมพร*"),COUNTIF(B84,"*เชียงราย*"),COUNTIF(B84,"*ตรัง*"),COUNTIF(B84,"*นครนายก*"),COUNTIF(B84,"*ปราจีนบุรี*"),COUNTIF(B84,"*พัทลุง*"),COUNTIF(B84,"*ภูเก็ต*"),COUNTIF(B84,"*ยะลา*"),COUNTIF(B84,"*สกลนคร*"),COUNTIF(B84,"*สตูล*"),COUNTIF(B84,"*หนองคาย*"),COUNTIF(B84,"*สุราษฎร์ธานี*"),COUNTIF(B84,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B84,"*ตราด*"),COUNTIF(B84,"*นครพนม*"),COUNTIF(B84,"*นครศรีธรรมราช*"),COUNTIF(B84,"*นราธิวาส*"),COUNTIF(B84,"*บึงกาฬ*"),COUNTIF(B84,"*พังงา*"),COUNTIF(B84,"*ระนอง*"),COUNTIF(B84,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM84">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>31239469.100000001</v>
       </c>
-    </row>
-    <row r="85" spans="1:39">
+      <c r="AN84">
+        <v>9383.7999999999993</v>
+      </c>
+    </row>
+    <row r="85" spans="1:40">
       <c r="A85" t="s">
         <v>136</v>
       </c>
@@ -14491,16 +14665,18 @@
         <v>300000</v>
       </c>
       <c r="AL85">
-        <f>IF(OR(COUNTIF(B85,"*กระบี่*"),COUNTIF(B85,"*จันทบุรี*"),COUNTIF(B85,"*ชุมพร*"),COUNTIF(B85,"*เชียงราย*"),COUNTIF(B85,"*ตรัง*"),COUNTIF(B85,"*นครนายก*"),COUNTIF(B85,"*ปราจีนบุรี*"),COUNTIF(B85,"*พัทลุง*"),COUNTIF(B85,"*ภูเก็ต*"),COUNTIF(B85,"*ยะลา*"),COUNTIF(B85,"*สกลนคร*"),COUNTIF(B85,"*สตูล*"),COUNTIF(B85,"*หนองคาย*"),COUNTIF(B85,"*สุราษฎร์ธานี*"),COUNTIF(B85,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B85,"*ตราด*"),COUNTIF(B85,"*นครพนม*"),COUNTIF(B85,"*นครศรีธรรมราช*"),COUNTIF(B85,"*นราธิวาส*"),COUNTIF(B85,"*บึงกาฬ*"),COUNTIF(B85,"*พังงา*"),COUNTIF(B85,"*ระนอง*"),COUNTIF(B85,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM85">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>36501247.039999999</v>
       </c>
-    </row>
-    <row r="86" spans="1:39">
+      <c r="AN85">
+        <v>4266.5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:40">
       <c r="A86" t="s">
         <v>134</v>
       </c>
@@ -14623,16 +14799,18 @@
         <v>0</v>
       </c>
       <c r="AL86">
-        <f>IF(OR(COUNTIF(B86,"*กระบี่*"),COUNTIF(B86,"*จันทบุรี*"),COUNTIF(B86,"*ชุมพร*"),COUNTIF(B86,"*เชียงราย*"),COUNTIF(B86,"*ตรัง*"),COUNTIF(B86,"*นครนายก*"),COUNTIF(B86,"*ปราจีนบุรี*"),COUNTIF(B86,"*พัทลุง*"),COUNTIF(B86,"*ภูเก็ต*"),COUNTIF(B86,"*ยะลา*"),COUNTIF(B86,"*สกลนคร*"),COUNTIF(B86,"*สตูล*"),COUNTIF(B86,"*หนองคาย*"),COUNTIF(B86,"*สุราษฎร์ธานี*"),COUNTIF(B86,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B86,"*ตราด*"),COUNTIF(B86,"*นครพนม*"),COUNTIF(B86,"*นครศรีธรรมราช*"),COUNTIF(B86,"*นราธิวาส*"),COUNTIF(B86,"*บึงกาฬ*"),COUNTIF(B86,"*พังงา*"),COUNTIF(B86,"*ระนอง*"),COUNTIF(B86,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM86">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>22397913</v>
       </c>
-    </row>
-    <row r="87" spans="1:39">
+      <c r="AN86">
+        <v>4415.2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:40">
       <c r="A87" t="s">
         <v>134</v>
       </c>
@@ -14755,16 +14933,18 @@
         <v>300000</v>
       </c>
       <c r="AL87">
-        <f>IF(OR(COUNTIF(B87,"*กระบี่*"),COUNTIF(B87,"*จันทบุรี*"),COUNTIF(B87,"*ชุมพร*"),COUNTIF(B87,"*เชียงราย*"),COUNTIF(B87,"*ตรัง*"),COUNTIF(B87,"*นครนายก*"),COUNTIF(B87,"*ปราจีนบุรี*"),COUNTIF(B87,"*พัทลุง*"),COUNTIF(B87,"*ภูเก็ต*"),COUNTIF(B87,"*ยะลา*"),COUNTIF(B87,"*สกลนคร*"),COUNTIF(B87,"*สตูล*"),COUNTIF(B87,"*หนองคาย*"),COUNTIF(B87,"*สุราษฎร์ธานี*"),COUNTIF(B87,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B87,"*ตราด*"),COUNTIF(B87,"*นครพนม*"),COUNTIF(B87,"*นครศรีธรรมราช*"),COUNTIF(B87,"*นราธิวาส*"),COUNTIF(B87,"*บึงกาฬ*"),COUNTIF(B87,"*พังงา*"),COUNTIF(B87,"*ระนอง*"),COUNTIF(B87,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM87">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>34308861</v>
       </c>
-    </row>
-    <row r="88" spans="1:39">
+      <c r="AN87">
+        <v>4975.3999999999996</v>
+      </c>
+    </row>
+    <row r="88" spans="1:40">
       <c r="A88" t="s">
         <v>134</v>
       </c>
@@ -14887,16 +15067,18 @@
         <v>0</v>
       </c>
       <c r="AL88">
-        <f>IF(OR(COUNTIF(B88,"*กระบี่*"),COUNTIF(B88,"*จันทบุรี*"),COUNTIF(B88,"*ชุมพร*"),COUNTIF(B88,"*เชียงราย*"),COUNTIF(B88,"*ตรัง*"),COUNTIF(B88,"*นครนายก*"),COUNTIF(B88,"*ปราจีนบุรี*"),COUNTIF(B88,"*พัทลุง*"),COUNTIF(B88,"*ภูเก็ต*"),COUNTIF(B88,"*ยะลา*"),COUNTIF(B88,"*สกลนคร*"),COUNTIF(B88,"*สตูล*"),COUNTIF(B88,"*หนองคาย*"),COUNTIF(B88,"*สุราษฎร์ธานี*"),COUNTIF(B88,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B88,"*ตราด*"),COUNTIF(B88,"*นครพนม*"),COUNTIF(B88,"*นครศรีธรรมราช*"),COUNTIF(B88,"*นราธิวาส*"),COUNTIF(B88,"*บึงกาฬ*"),COUNTIF(B88,"*พังงา*"),COUNTIF(B88,"*ระนอง*"),COUNTIF(B88,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM88">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>115835052</v>
       </c>
-    </row>
-    <row r="89" spans="1:39">
+      <c r="AN88">
+        <v>6942.8</v>
+      </c>
+    </row>
+    <row r="89" spans="1:40">
       <c r="A89" t="s">
         <v>134</v>
       </c>
@@ -15019,16 +15201,18 @@
         <v>0</v>
       </c>
       <c r="AL89">
-        <f>IF(OR(COUNTIF(B89,"*กระบี่*"),COUNTIF(B89,"*จันทบุรี*"),COUNTIF(B89,"*ชุมพร*"),COUNTIF(B89,"*เชียงราย*"),COUNTIF(B89,"*ตรัง*"),COUNTIF(B89,"*นครนายก*"),COUNTIF(B89,"*ปราจีนบุรี*"),COUNTIF(B89,"*พัทลุง*"),COUNTIF(B89,"*ภูเก็ต*"),COUNTIF(B89,"*ยะลา*"),COUNTIF(B89,"*สกลนคร*"),COUNTIF(B89,"*สตูล*"),COUNTIF(B89,"*หนองคาย*"),COUNTIF(B89,"*สุราษฎร์ธานี*"),COUNTIF(B89,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B89,"*ตราด*"),COUNTIF(B89,"*นครพนม*"),COUNTIF(B89,"*นครศรีธรรมราช*"),COUNTIF(B89,"*นราธิวาส*"),COUNTIF(B89,"*บึงกาฬ*"),COUNTIF(B89,"*พังงา*"),COUNTIF(B89,"*ระนอง*"),COUNTIF(B89,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM89">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>48262457.539999999</v>
       </c>
-    </row>
-    <row r="90" spans="1:39">
+      <c r="AN89">
+        <v>5068</v>
+      </c>
+    </row>
+    <row r="90" spans="1:40">
       <c r="A90" t="s">
         <v>134</v>
       </c>
@@ -15151,16 +15335,18 @@
         <v>0</v>
       </c>
       <c r="AL90">
-        <f>IF(OR(COUNTIF(B90,"*กระบี่*"),COUNTIF(B90,"*จันทบุรี*"),COUNTIF(B90,"*ชุมพร*"),COUNTIF(B90,"*เชียงราย*"),COUNTIF(B90,"*ตรัง*"),COUNTIF(B90,"*นครนายก*"),COUNTIF(B90,"*ปราจีนบุรี*"),COUNTIF(B90,"*พัทลุง*"),COUNTIF(B90,"*ภูเก็ต*"),COUNTIF(B90,"*ยะลา*"),COUNTIF(B90,"*สกลนคร*"),COUNTIF(B90,"*สตูล*"),COUNTIF(B90,"*หนองคาย*"),COUNTIF(B90,"*สุราษฎร์ธานี*"),COUNTIF(B90,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B90,"*ตราด*"),COUNTIF(B90,"*นครพนม*"),COUNTIF(B90,"*นครศรีธรรมราช*"),COUNTIF(B90,"*นราธิวาส*"),COUNTIF(B90,"*บึงกาฬ*"),COUNTIF(B90,"*พังงา*"),COUNTIF(B90,"*ระนอง*"),COUNTIF(B90,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM90">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>20132405.359999999</v>
       </c>
-    </row>
-    <row r="91" spans="1:39">
+      <c r="AN90">
+        <v>5280</v>
+      </c>
+    </row>
+    <row r="91" spans="1:40">
       <c r="A91" t="s">
         <v>118</v>
       </c>
@@ -15283,20 +15469,22 @@
         <v>0</v>
       </c>
       <c r="AL91">
-        <f>IF(OR(COUNTIF(B91,"*กระบี่*"),COUNTIF(B91,"*จันทบุรี*"),COUNTIF(B91,"*ชุมพร*"),COUNTIF(B91,"*เชียงราย*"),COUNTIF(B91,"*ตรัง*"),COUNTIF(B91,"*นครนายก*"),COUNTIF(B91,"*ปราจีนบุรี*"),COUNTIF(B91,"*พัทลุง*"),COUNTIF(B91,"*ภูเก็ต*"),COUNTIF(B91,"*ยะลา*"),COUNTIF(B91,"*สกลนคร*"),COUNTIF(B91,"*สตูล*"),COUNTIF(B91,"*หนองคาย*"),COUNTIF(B91,"*สุราษฎร์ธานี*"),COUNTIF(B91,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B91,"*ตราด*"),COUNTIF(B91,"*นครพนม*"),COUNTIF(B91,"*นครศรีธรรมราช*"),COUNTIF(B91,"*นราธิวาส*"),COUNTIF(B91,"*บึงกาฬ*"),COUNTIF(B91,"*พังงา*"),COUNTIF(B91,"*ระนอง*"),COUNTIF(B91,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM91">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>23887668.25</v>
       </c>
-    </row>
-    <row r="92" spans="1:39">
+      <c r="AN91">
+        <v>2332.5</v>
+      </c>
+    </row>
+    <row r="92" spans="1:40">
       <c r="A92" t="s">
         <v>129</v>
       </c>
-      <c r="B92" s="82" t="s">
+      <c r="B92" t="s">
         <v>144</v>
       </c>
       <c r="C92" s="39">
@@ -15313,73 +15501,73 @@
       <c r="F92">
         <v>182203618</v>
       </c>
-      <c r="G92" s="82">
+      <c r="G92">
         <v>2.5269333333333335</v>
       </c>
-      <c r="H92" s="82">
+      <c r="H92">
         <v>485.98199999999997</v>
       </c>
-      <c r="I92" s="82">
+      <c r="I92">
         <v>1</v>
       </c>
-      <c r="J92" s="82">
+      <c r="J92">
         <v>8</v>
       </c>
-      <c r="K92" s="82">
+      <c r="K92">
         <v>3.2666666666666666</v>
       </c>
-      <c r="L92" s="82">
+      <c r="L92">
         <v>3.5</v>
       </c>
-      <c r="M92" s="82">
+      <c r="M92">
         <v>5</v>
       </c>
-      <c r="N92" s="82">
+      <c r="N92">
         <v>27.712</v>
       </c>
-      <c r="O92" s="82">
+      <c r="O92">
         <v>2</v>
       </c>
-      <c r="P92" s="82">
+      <c r="P92">
         <v>8</v>
       </c>
-      <c r="Q92" s="82">
+      <c r="Q92">
         <v>4.875</v>
       </c>
-      <c r="R92" s="82">
+      <c r="R92">
         <v>3.5</v>
       </c>
-      <c r="S92" s="82">
+      <c r="S92">
         <v>5.125</v>
       </c>
-      <c r="T92" s="82">
-        <v>0</v>
-      </c>
-      <c r="U92" s="82">
+      <c r="T92">
+        <v>0</v>
+      </c>
+      <c r="U92">
         <v>10201</v>
       </c>
-      <c r="V92" s="82">
+      <c r="V92">
         <v>128266.6</v>
       </c>
-      <c r="W92" s="82">
+      <c r="W92">
         <v>2034.9</v>
       </c>
-      <c r="X92" s="82">
+      <c r="X92">
         <v>109588.20400000001</v>
       </c>
-      <c r="Y92" s="82">
+      <c r="Y92">
         <v>90798.187999999995</v>
       </c>
-      <c r="Z92" s="82">
+      <c r="Z92">
         <v>117.93882513258733</v>
       </c>
-      <c r="AA92" s="82">
+      <c r="AA92">
         <v>44.364150129287701</v>
       </c>
-      <c r="AB92" s="82">
+      <c r="AB92">
         <v>-1.4132145275342572E-2</v>
       </c>
-      <c r="AC92" s="82">
+      <c r="AC92">
         <v>13.239974166133312</v>
       </c>
       <c r="AD92">
@@ -15415,20 +15603,22 @@
         <v>300000</v>
       </c>
       <c r="AL92">
-        <f>IF(OR(COUNTIF(B92,"*กระบี่*"),COUNTIF(B92,"*จันทบุรี*"),COUNTIF(B92,"*ชุมพร*"),COUNTIF(B92,"*เชียงราย*"),COUNTIF(B92,"*ตรัง*"),COUNTIF(B92,"*นครนายก*"),COUNTIF(B92,"*ปราจีนบุรี*"),COUNTIF(B92,"*พัทลุง*"),COUNTIF(B92,"*ภูเก็ต*"),COUNTIF(B92,"*ยะลา*"),COUNTIF(B92,"*สกลนคร*"),COUNTIF(B92,"*สตูล*"),COUNTIF(B92,"*หนองคาย*"),COUNTIF(B92,"*สุราษฎร์ธานี*"),COUNTIF(B92,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B92,"*ตราด*"),COUNTIF(B92,"*นครพนม*"),COUNTIF(B92,"*นครศรีธรรมราช*"),COUNTIF(B92,"*นราธิวาส*"),COUNTIF(B92,"*บึงกาฬ*"),COUNTIF(B92,"*พังงา*"),COUNTIF(B92,"*ระนอง*"),COUNTIF(B92,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM92">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>30781563.02</v>
       </c>
-    </row>
-    <row r="93" spans="1:39">
+      <c r="AN92">
+        <v>7419</v>
+      </c>
+    </row>
+    <row r="93" spans="1:40">
       <c r="A93" t="s">
         <v>129</v>
       </c>
-      <c r="B93" s="82" t="s">
+      <c r="B93" t="s">
         <v>145</v>
       </c>
       <c r="C93" s="39">
@@ -15445,73 +15635,73 @@
       <c r="F93">
         <v>264584953</v>
       </c>
-      <c r="G93" s="82">
+      <c r="G93">
         <v>2.7022727272727276</v>
       </c>
-      <c r="H93" s="82">
+      <c r="H93">
         <v>332.12099999999998</v>
       </c>
-      <c r="I93" s="82">
+      <c r="I93">
         <v>1</v>
       </c>
-      <c r="J93" s="82">
+      <c r="J93">
         <v>8</v>
       </c>
-      <c r="K93" s="82">
+      <c r="K93">
         <v>2.8181818181818183</v>
       </c>
-      <c r="L93" s="82">
+      <c r="L93">
         <v>4.3550000000000004</v>
       </c>
-      <c r="M93" s="82">
+      <c r="M93">
         <v>6.25</v>
       </c>
-      <c r="N93" s="82">
+      <c r="N93">
         <v>3.6970000000000001</v>
       </c>
-      <c r="O93" s="82">
+      <c r="O93">
         <v>4</v>
       </c>
-      <c r="P93" s="82">
+      <c r="P93">
         <v>8</v>
       </c>
-      <c r="Q93" s="82">
+      <c r="Q93">
         <v>5</v>
       </c>
-      <c r="R93" s="82">
+      <c r="R93">
         <v>3.5</v>
       </c>
-      <c r="S93" s="82">
+      <c r="S93">
         <v>5</v>
       </c>
-      <c r="T93" s="82">
-        <v>0</v>
-      </c>
-      <c r="U93" s="82">
-        <v>0</v>
-      </c>
-      <c r="V93" s="82">
+      <c r="T93">
+        <v>0</v>
+      </c>
+      <c r="U93">
+        <v>0</v>
+      </c>
+      <c r="V93">
         <v>63853.649999999994</v>
       </c>
-      <c r="W93" s="82">
+      <c r="W93">
         <v>1675</v>
       </c>
-      <c r="X93" s="82">
+      <c r="X93">
         <v>135061.19</v>
       </c>
-      <c r="Y93" s="82">
+      <c r="Y93">
         <v>106902.356</v>
       </c>
-      <c r="Z93" s="82">
+      <c r="Z93">
         <v>146.99492059378974</v>
       </c>
-      <c r="AA93" s="82">
+      <c r="AA93">
         <v>171.21254993214887</v>
       </c>
-      <c r="AB93" s="82">
+      <c r="AB93">
         <v>7.4021965588661601E-2</v>
       </c>
-      <c r="AC93" s="82">
+      <c r="AC93">
         <v>12.522181304120181</v>
       </c>
       <c r="AD93">
@@ -15547,16 +15737,18 @@
         <v>0</v>
       </c>
       <c r="AL93">
-        <f>IF(OR(COUNTIF(B93,"*กระบี่*"),COUNTIF(B93,"*จันทบุรี*"),COUNTIF(B93,"*ชุมพร*"),COUNTIF(B93,"*เชียงราย*"),COUNTIF(B93,"*ตรัง*"),COUNTIF(B93,"*นครนายก*"),COUNTIF(B93,"*ปราจีนบุรี*"),COUNTIF(B93,"*พัทลุง*"),COUNTIF(B93,"*ภูเก็ต*"),COUNTIF(B93,"*ยะลา*"),COUNTIF(B93,"*สกลนคร*"),COUNTIF(B93,"*สตูล*"),COUNTIF(B93,"*หนองคาย*"),COUNTIF(B93,"*สุราษฎร์ธานี*"),COUNTIF(B93,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B93,"*ตราด*"),COUNTIF(B93,"*นครพนม*"),COUNTIF(B93,"*นครศรีธรรมราช*"),COUNTIF(B93,"*นราธิวาส*"),COUNTIF(B93,"*บึงกาฬ*"),COUNTIF(B93,"*พังงา*"),COUNTIF(B93,"*ระนอง*"),COUNTIF(B93,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM93">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>31476285.129999999</v>
       </c>
-    </row>
-    <row r="94" spans="1:39">
+      <c r="AN93">
+        <v>6151.5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:40">
       <c r="A94" t="s">
         <v>136</v>
       </c>
@@ -15679,16 +15871,18 @@
         <v>0</v>
       </c>
       <c r="AL94">
-        <f>IF(OR(COUNTIF(B94,"*กระบี่*"),COUNTIF(B94,"*จันทบุรี*"),COUNTIF(B94,"*ชุมพร*"),COUNTIF(B94,"*เชียงราย*"),COUNTIF(B94,"*ตรัง*"),COUNTIF(B94,"*นครนายก*"),COUNTIF(B94,"*ปราจีนบุรี*"),COUNTIF(B94,"*พัทลุง*"),COUNTIF(B94,"*ภูเก็ต*"),COUNTIF(B94,"*ยะลา*"),COUNTIF(B94,"*สกลนคร*"),COUNTIF(B94,"*สตูล*"),COUNTIF(B94,"*หนองคาย*"),COUNTIF(B94,"*สุราษฎร์ธานี*"),COUNTIF(B94,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B94,"*ตราด*"),COUNTIF(B94,"*นครพนม*"),COUNTIF(B94,"*นครศรีธรรมราช*"),COUNTIF(B94,"*นราธิวาส*"),COUNTIF(B94,"*บึงกาฬ*"),COUNTIF(B94,"*พังงา*"),COUNTIF(B94,"*ระนอง*"),COUNTIF(B94,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM94">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>16316511</v>
       </c>
-    </row>
-    <row r="95" spans="1:39">
+      <c r="AN94">
+        <v>5807.8</v>
+      </c>
+    </row>
+    <row r="95" spans="1:40">
       <c r="A95" t="s">
         <v>129</v>
       </c>
@@ -15811,16 +16005,18 @@
         <v>300000</v>
       </c>
       <c r="AL95">
-        <f>IF(OR(COUNTIF(B95,"*กระบี่*"),COUNTIF(B95,"*จันทบุรี*"),COUNTIF(B95,"*ชุมพร*"),COUNTIF(B95,"*เชียงราย*"),COUNTIF(B95,"*ตรัง*"),COUNTIF(B95,"*นครนายก*"),COUNTIF(B95,"*ปราจีนบุรี*"),COUNTIF(B95,"*พัทลุง*"),COUNTIF(B95,"*ภูเก็ต*"),COUNTIF(B95,"*ยะลา*"),COUNTIF(B95,"*สกลนคร*"),COUNTIF(B95,"*สตูล*"),COUNTIF(B95,"*หนองคาย*"),COUNTIF(B95,"*สุราษฎร์ธานี*"),COUNTIF(B95,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B95,"*ตราด*"),COUNTIF(B95,"*นครพนม*"),COUNTIF(B95,"*นครศรีธรรมราช*"),COUNTIF(B95,"*นราธิวาส*"),COUNTIF(B95,"*บึงกาฬ*"),COUNTIF(B95,"*พังงา*"),COUNTIF(B95,"*ระนอง*"),COUNTIF(B95,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM95">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>16720167.5</v>
       </c>
-    </row>
-    <row r="96" spans="1:39">
+      <c r="AN95">
+        <v>6656.7</v>
+      </c>
+    </row>
+    <row r="96" spans="1:40">
       <c r="A96" t="s">
         <v>136</v>
       </c>
@@ -15943,16 +16139,18 @@
         <v>0</v>
       </c>
       <c r="AL96">
-        <f>IF(OR(COUNTIF(B96,"*กระบี่*"),COUNTIF(B96,"*จันทบุรี*"),COUNTIF(B96,"*ชุมพร*"),COUNTIF(B96,"*เชียงราย*"),COUNTIF(B96,"*ตรัง*"),COUNTIF(B96,"*นครนายก*"),COUNTIF(B96,"*ปราจีนบุรี*"),COUNTIF(B96,"*พัทลุง*"),COUNTIF(B96,"*ภูเก็ต*"),COUNTIF(B96,"*ยะลา*"),COUNTIF(B96,"*สกลนคร*"),COUNTIF(B96,"*สตูล*"),COUNTIF(B96,"*หนองคาย*"),COUNTIF(B96,"*สุราษฎร์ธานี*"),COUNTIF(B96,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B96,"*ตราด*"),COUNTIF(B96,"*นครพนม*"),COUNTIF(B96,"*นครศรีธรรมราช*"),COUNTIF(B96,"*นราธิวาส*"),COUNTIF(B96,"*บึงกาฬ*"),COUNTIF(B96,"*พังงา*"),COUNTIF(B96,"*ระนอง*"),COUNTIF(B96,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM96">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>40211709</v>
       </c>
-    </row>
-    <row r="97" spans="1:39">
+      <c r="AN96">
+        <v>3988.9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:40">
       <c r="A97" t="s">
         <v>129</v>
       </c>
@@ -16075,16 +16273,18 @@
         <v>600000</v>
       </c>
       <c r="AL97">
-        <f>IF(OR(COUNTIF(B97,"*กระบี่*"),COUNTIF(B97,"*จันทบุรี*"),COUNTIF(B97,"*ชุมพร*"),COUNTIF(B97,"*เชียงราย*"),COUNTIF(B97,"*ตรัง*"),COUNTIF(B97,"*นครนายก*"),COUNTIF(B97,"*ปราจีนบุรี*"),COUNTIF(B97,"*พัทลุง*"),COUNTIF(B97,"*ภูเก็ต*"),COUNTIF(B97,"*ยะลา*"),COUNTIF(B97,"*สกลนคร*"),COUNTIF(B97,"*สตูล*"),COUNTIF(B97,"*หนองคาย*"),COUNTIF(B97,"*สุราษฎร์ธานี*"),COUNTIF(B97,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B97,"*ตราด*"),COUNTIF(B97,"*นครพนม*"),COUNTIF(B97,"*นครศรีธรรมราช*"),COUNTIF(B97,"*นราธิวาส*"),COUNTIF(B97,"*บึงกาฬ*"),COUNTIF(B97,"*พังงา*"),COUNTIF(B97,"*ระนอง*"),COUNTIF(B97,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AM97">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>16859979.280000001</v>
       </c>
-    </row>
-    <row r="98" spans="1:39">
+      <c r="AN97">
+        <v>2534.5</v>
+      </c>
+    </row>
+    <row r="98" spans="1:40">
       <c r="A98" t="s">
         <v>129</v>
       </c>
@@ -16207,7 +16407,7 @@
         <v>300000</v>
       </c>
       <c r="AL98">
-        <f>IF(OR(COUNTIF(B98,"*กระบี่*"),COUNTIF(B98,"*จันทบุรี*"),COUNTIF(B98,"*ชุมพร*"),COUNTIF(B98,"*เชียงราย*"),COUNTIF(B98,"*ตรัง*"),COUNTIF(B98,"*นครนายก*"),COUNTIF(B98,"*ปราจีนบุรี*"),COUNTIF(B98,"*พัทลุง*"),COUNTIF(B98,"*ภูเก็ต*"),COUNTIF(B98,"*ยะลา*"),COUNTIF(B98,"*สกลนคร*"),COUNTIF(B98,"*สตูล*"),COUNTIF(B98,"*หนองคาย*"),COUNTIF(B98,"*สุราษฎร์ธานี*"),COUNTIF(B98,"*ปัตตานี*")),2,
+        <f t="shared" ref="AL98:AL105" si="3">IF(OR(COUNTIF(B98,"*กระบี่*"),COUNTIF(B98,"*จันทบุรี*"),COUNTIF(B98,"*ชุมพร*"),COUNTIF(B98,"*เชียงราย*"),COUNTIF(B98,"*ตรัง*"),COUNTIF(B98,"*นครนายก*"),COUNTIF(B98,"*ปราจีนบุรี*"),COUNTIF(B98,"*พัทลุง*"),COUNTIF(B98,"*ภูเก็ต*"),COUNTIF(B98,"*ยะลา*"),COUNTIF(B98,"*สกลนคร*"),COUNTIF(B98,"*สตูล*"),COUNTIF(B98,"*หนองคาย*"),COUNTIF(B98,"*สุราษฎร์ธานี*"),COUNTIF(B98,"*ปัตตานี*")),2,
 IF(OR(COUNTIF(B98,"*ตราด*"),COUNTIF(B98,"*นครพนม*"),COUNTIF(B98,"*นครศรีธรรมราช*"),COUNTIF(B98,"*นราธิวาส*"),COUNTIF(B98,"*บึงกาฬ*"),COUNTIF(B98,"*พังงา*"),COUNTIF(B98,"*ระนอง*"),COUNTIF(B98,"*สงขลา*")),4,0))</f>
         <v>0</v>
       </c>
@@ -16215,8 +16415,11 @@
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>16130059</v>
       </c>
-    </row>
-    <row r="99" spans="1:39">
+      <c r="AN98">
+        <v>4812.3999999999996</v>
+      </c>
+    </row>
+    <row r="99" spans="1:40">
       <c r="A99" t="s">
         <v>151</v>
       </c>
@@ -16339,16 +16542,18 @@
         <v>600000</v>
       </c>
       <c r="AL99">
-        <f>IF(OR(COUNTIF(B99,"*กระบี่*"),COUNTIF(B99,"*จันทบุรี*"),COUNTIF(B99,"*ชุมพร*"),COUNTIF(B99,"*เชียงราย*"),COUNTIF(B99,"*ตรัง*"),COUNTIF(B99,"*นครนายก*"),COUNTIF(B99,"*ปราจีนบุรี*"),COUNTIF(B99,"*พัทลุง*"),COUNTIF(B99,"*ภูเก็ต*"),COUNTIF(B99,"*ยะลา*"),COUNTIF(B99,"*สกลนคร*"),COUNTIF(B99,"*สตูล*"),COUNTIF(B99,"*หนองคาย*"),COUNTIF(B99,"*สุราษฎร์ธานี*"),COUNTIF(B99,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B99,"*ตราด*"),COUNTIF(B99,"*นครพนม*"),COUNTIF(B99,"*นครศรีธรรมราช*"),COUNTIF(B99,"*นราธิวาส*"),COUNTIF(B99,"*บึงกาฬ*"),COUNTIF(B99,"*พังงา*"),COUNTIF(B99,"*ระนอง*"),COUNTIF(B99,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AM99">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>17347616.379999999</v>
       </c>
-    </row>
-    <row r="100" spans="1:39">
+      <c r="AN99">
+        <v>9799</v>
+      </c>
+    </row>
+    <row r="100" spans="1:40">
       <c r="A100" t="s">
         <v>151</v>
       </c>
@@ -16471,16 +16676,18 @@
         <v>0</v>
       </c>
       <c r="AL100">
-        <f>IF(OR(COUNTIF(B100,"*กระบี่*"),COUNTIF(B100,"*จันทบุรี*"),COUNTIF(B100,"*ชุมพร*"),COUNTIF(B100,"*เชียงราย*"),COUNTIF(B100,"*ตรัง*"),COUNTIF(B100,"*นครนายก*"),COUNTIF(B100,"*ปราจีนบุรี*"),COUNTIF(B100,"*พัทลุง*"),COUNTIF(B100,"*ภูเก็ต*"),COUNTIF(B100,"*ยะลา*"),COUNTIF(B100,"*สกลนคร*"),COUNTIF(B100,"*สตูล*"),COUNTIF(B100,"*หนองคาย*"),COUNTIF(B100,"*สุราษฎร์ธานี*"),COUNTIF(B100,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B100,"*ตราด*"),COUNTIF(B100,"*นครพนม*"),COUNTIF(B100,"*นครศรีธรรมราช*"),COUNTIF(B100,"*นราธิวาส*"),COUNTIF(B100,"*บึงกาฬ*"),COUNTIF(B100,"*พังงา*"),COUNTIF(B100,"*ระนอง*"),COUNTIF(B100,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="3"/>
         <v>2</v>
       </c>
       <c r="AM100">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>61274963.369999997</v>
       </c>
-    </row>
-    <row r="101" spans="1:39">
+      <c r="AN100">
+        <v>5111</v>
+      </c>
+    </row>
+    <row r="101" spans="1:40">
       <c r="A101" t="s">
         <v>151</v>
       </c>
@@ -16603,16 +16810,18 @@
         <v>300000</v>
       </c>
       <c r="AL101">
-        <f>IF(OR(COUNTIF(B101,"*กระบี่*"),COUNTIF(B101,"*จันทบุรี*"),COUNTIF(B101,"*ชุมพร*"),COUNTIF(B101,"*เชียงราย*"),COUNTIF(B101,"*ตรัง*"),COUNTIF(B101,"*นครนายก*"),COUNTIF(B101,"*ปราจีนบุรี*"),COUNTIF(B101,"*พัทลุง*"),COUNTIF(B101,"*ภูเก็ต*"),COUNTIF(B101,"*ยะลา*"),COUNTIF(B101,"*สกลนคร*"),COUNTIF(B101,"*สตูล*"),COUNTIF(B101,"*หนองคาย*"),COUNTIF(B101,"*สุราษฎร์ธานี*"),COUNTIF(B101,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B101,"*ตราด*"),COUNTIF(B101,"*นครพนม*"),COUNTIF(B101,"*นครศรีธรรมราช*"),COUNTIF(B101,"*นราธิวาส*"),COUNTIF(B101,"*บึงกาฬ*"),COUNTIF(B101,"*พังงา*"),COUNTIF(B101,"*ระนอง*"),COUNTIF(B101,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="3"/>
         <v>2</v>
       </c>
       <c r="AM101">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>24252916.210000001</v>
       </c>
-    </row>
-    <row r="102" spans="1:39">
+      <c r="AN101">
+        <v>5579</v>
+      </c>
+    </row>
+    <row r="102" spans="1:40">
       <c r="A102" t="s">
         <v>151</v>
       </c>
@@ -16729,16 +16938,18 @@
         <v>300000</v>
       </c>
       <c r="AL102">
-        <f>IF(OR(COUNTIF(B102,"*กระบี่*"),COUNTIF(B102,"*จันทบุรี*"),COUNTIF(B102,"*ชุมพร*"),COUNTIF(B102,"*เชียงราย*"),COUNTIF(B102,"*ตรัง*"),COUNTIF(B102,"*นครนายก*"),COUNTIF(B102,"*ปราจีนบุรี*"),COUNTIF(B102,"*พัทลุง*"),COUNTIF(B102,"*ภูเก็ต*"),COUNTIF(B102,"*ยะลา*"),COUNTIF(B102,"*สกลนคร*"),COUNTIF(B102,"*สตูล*"),COUNTIF(B102,"*หนองคาย*"),COUNTIF(B102,"*สุราษฎร์ธานี*"),COUNTIF(B102,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B102,"*ตราด*"),COUNTIF(B102,"*นครพนม*"),COUNTIF(B102,"*นครศรีธรรมราช*"),COUNTIF(B102,"*นราธิวาส*"),COUNTIF(B102,"*บึงกาฬ*"),COUNTIF(B102,"*พังงา*"),COUNTIF(B102,"*ระนอง*"),COUNTIF(B102,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="3"/>
         <v>4</v>
       </c>
       <c r="AM102">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>11182835</v>
       </c>
-    </row>
-    <row r="103" spans="1:39">
+      <c r="AN102">
+        <v>4746</v>
+      </c>
+    </row>
+    <row r="103" spans="1:40">
       <c r="A103" t="s">
         <v>151</v>
       </c>
@@ -16861,16 +17072,18 @@
         <v>600000</v>
       </c>
       <c r="AL103">
-        <f>IF(OR(COUNTIF(B103,"*กระบี่*"),COUNTIF(B103,"*จันทบุรี*"),COUNTIF(B103,"*ชุมพร*"),COUNTIF(B103,"*เชียงราย*"),COUNTIF(B103,"*ตรัง*"),COUNTIF(B103,"*นครนายก*"),COUNTIF(B103,"*ปราจีนบุรี*"),COUNTIF(B103,"*พัทลุง*"),COUNTIF(B103,"*ภูเก็ต*"),COUNTIF(B103,"*ยะลา*"),COUNTIF(B103,"*สกลนคร*"),COUNTIF(B103,"*สตูล*"),COUNTIF(B103,"*หนองคาย*"),COUNTIF(B103,"*สุราษฎร์ธานี*"),COUNTIF(B103,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B103,"*ตราด*"),COUNTIF(B103,"*นครพนม*"),COUNTIF(B103,"*นครศรีธรรมราช*"),COUNTIF(B103,"*นราธิวาส*"),COUNTIF(B103,"*บึงกาฬ*"),COUNTIF(B103,"*พังงา*"),COUNTIF(B103,"*ระนอง*"),COUNTIF(B103,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="3"/>
         <v>4</v>
       </c>
       <c r="AM103">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>15897455.4</v>
       </c>
-    </row>
-    <row r="104" spans="1:39">
+      <c r="AN103">
+        <v>5868</v>
+      </c>
+    </row>
+    <row r="104" spans="1:40">
       <c r="A104" t="s">
         <v>151</v>
       </c>
@@ -16993,16 +17206,18 @@
         <v>0</v>
       </c>
       <c r="AL104">
-        <f>IF(OR(COUNTIF(B104,"*กระบี่*"),COUNTIF(B104,"*จันทบุรี*"),COUNTIF(B104,"*ชุมพร*"),COUNTIF(B104,"*เชียงราย*"),COUNTIF(B104,"*ตรัง*"),COUNTIF(B104,"*นครนายก*"),COUNTIF(B104,"*ปราจีนบุรี*"),COUNTIF(B104,"*พัทลุง*"),COUNTIF(B104,"*ภูเก็ต*"),COUNTIF(B104,"*ยะลา*"),COUNTIF(B104,"*สกลนคร*"),COUNTIF(B104,"*สตูล*"),COUNTIF(B104,"*หนองคาย*"),COUNTIF(B104,"*สุราษฎร์ธานี*"),COUNTIF(B104,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B104,"*ตราด*"),COUNTIF(B104,"*นครพนม*"),COUNTIF(B104,"*นครศรีธรรมราช*"),COUNTIF(B104,"*นราธิวาส*"),COUNTIF(B104,"*บึงกาฬ*"),COUNTIF(B104,"*พังงา*"),COUNTIF(B104,"*ระนอง*"),COUNTIF(B104,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="3"/>
         <v>2</v>
       </c>
       <c r="AM104">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>9945873</v>
       </c>
-    </row>
-    <row r="105" spans="1:39">
+      <c r="AN104">
+        <v>3575.9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:40">
       <c r="A105" t="s">
         <v>136</v>
       </c>
@@ -17125,13 +17340,15 @@
         <v>0</v>
       </c>
       <c r="AL105">
-        <f>IF(OR(COUNTIF(B105,"*กระบี่*"),COUNTIF(B105,"*จันทบุรี*"),COUNTIF(B105,"*ชุมพร*"),COUNTIF(B105,"*เชียงราย*"),COUNTIF(B105,"*ตรัง*"),COUNTIF(B105,"*นครนายก*"),COUNTIF(B105,"*ปราจีนบุรี*"),COUNTIF(B105,"*พัทลุง*"),COUNTIF(B105,"*ภูเก็ต*"),COUNTIF(B105,"*ยะลา*"),COUNTIF(B105,"*สกลนคร*"),COUNTIF(B105,"*สตูล*"),COUNTIF(B105,"*หนองคาย*"),COUNTIF(B105,"*สุราษฎร์ธานี*"),COUNTIF(B105,"*ปัตตานี*")),2,
-IF(OR(COUNTIF(B105,"*ตราด*"),COUNTIF(B105,"*นครพนม*"),COUNTIF(B105,"*นครศรีธรรมราช*"),COUNTIF(B105,"*นราธิวาส*"),COUNTIF(B105,"*บึงกาฬ*"),COUNTIF(B105,"*พังงา*"),COUNTIF(B105,"*ระนอง*"),COUNTIF(B105,"*สงขลา*")),4,0))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AM105">
         <f>_xlfn.XLOOKUP(group_data_final[[#This Row],[depot_code]],C:C,แผน68!D:D)</f>
         <v>5580390.4299999997</v>
+      </c>
+      <c r="AN105">
+        <v>10544</v>
       </c>
     </row>
   </sheetData>
@@ -40132,13 +40349,13 @@
       <c r="A1" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="B1" s="78" t="s">
+      <c r="B1" s="76" t="s">
         <v>273</v>
       </c>
       <c r="C1" s="46" t="s">
         <v>274</v>
       </c>
-      <c r="D1" s="80" t="s">
+      <c r="D1" s="78" t="s">
         <v>275</v>
       </c>
     </row>
@@ -40146,11 +40363,11 @@
       <c r="A2" s="47" t="s">
         <v>276</v>
       </c>
-      <c r="B2" s="79"/>
+      <c r="B2" s="77"/>
       <c r="C2" s="47" t="s">
         <v>277</v>
       </c>
-      <c r="D2" s="81"/>
+      <c r="D2" s="79"/>
     </row>
     <row r="3" spans="1:4" ht="24">
       <c r="A3" s="50">
@@ -57207,7 +57424,7 @@
       <c r="A34" s="25" t="s">
         <v>511</v>
       </c>
-      <c r="B34" s="76" t="s">
+      <c r="B34" s="80" t="s">
         <v>479</v>
       </c>
     </row>
@@ -57215,7 +57432,7 @@
       <c r="A35" s="30" t="s">
         <v>512</v>
       </c>
-      <c r="B35" s="77"/>
+      <c r="B35" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>